<commit_message>
Thursday Aug 13: Logged and confirmed Team Ace HR (Row 119) and Xponentium (Row 120) Snowflake Lead NVites
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O118"/>
+  <dimension ref="A1:O120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -7495,7 +7495,7 @@
       </c>
       <c r="D104" s="29" t="inlineStr">
         <is>
-          <t>Bangalore (On-site F2F Drive)</t>
+          <t>Bengaluru (Electronic City Phase I Tech Hub)</t>
         </is>
       </c>
       <c r="E104" s="29" t="inlineStr">
@@ -7543,7 +7543,7 @@
       </c>
       <c r="N104" s="29" t="inlineStr">
         <is>
-          <t>Confirmation email sent on Wednesday Aug 12 @ 2:40 PM to Komal Pawar (komal-ganesh.pawar@db.com) confirming F2F interview drive participation on Saturday Aug 22 at DB Bangalore office.</t>
+          <t>Confirmation email sent on Wed Aug 12 to Komal Pawar (komal-ganesh.pawar@db.com) for Saturday Aug 22 F2F drive. Venue: Deutsche Bank Tech Hub, Electronic City Phase I, Doddathoguru, Bengaluru 560100.</t>
         </is>
       </c>
       <c r="O104" s="29" t="inlineStr">
@@ -8602,8 +8602,156 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="33.95" customHeight="1" s="20"/>
-    <row r="120" ht="33.95" customHeight="1" s="20"/>
+    <row r="119" ht="33.95" customHeight="1" s="20">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Team Ace HR LLP (Client Requisition)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Snowflake Lead | ETL | Data Warehousing</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Hyderabad (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H119" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct NVite)</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Snehlata D (Team Ace HR LLP)</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>9999123932</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 9-18 Yrs, 2+ Yrs Snowflake Lead, DWH, ELT Pipelines, CTEs, Stored Procedures, Data Governance, Data Quality, Immediate Joiner.</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>Direct recruiter NVite received from Snehlata D (Team Ace HR) on Thu Aug 13 @ 7:50 AM. Applied and confirmed for Snowflake Lead | ETL | DWH in Hyderabad.</t>
+        </is>
+      </c>
+      <c r="O119" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="33.95" customHeight="1" s="20">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Xponentium (Rating: 4.4/5.0 Stars)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Snowflake Developer</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Hyderabad, Bengaluru, Pune</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter NVite</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H120" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct NVite)</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Chanya Roheda</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Naukri Direct NVite</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 10-17 Yrs, Snowflake, DWH Architecture, dbt Transformations, Advanced SQL, Data Governance &amp; Security, Immediate to 21 days NP.</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>Direct recruiter NVite received from Chanya Roheda (Xponentium) on Thu Aug 13 @ 10:52 AM. Applied and confirmed for Snowflake Developer in Bengaluru/Hyderabad/Pune.</t>
+        </is>
+      </c>
+      <c r="O120" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="121" ht="33.95" customHeight="1" s="20"/>
     <row r="122" ht="33.95" customHeight="1" s="20"/>
     <row r="123" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 13: Logged Recex Data Architect (Row 121) - Graduation Not Required
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O120"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -8752,7 +8752,81 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="33.95" customHeight="1" s="20"/>
+    <row r="121" ht="33.95" customHeight="1" s="20">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Recex (Agency Requisition)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Data Architect</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Bengaluru, Delhi / NCR, Mumbai</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Naukri Direct Posting</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H121" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Graduation Not Required)</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Recex Hiring Team</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>98% Match. Requirements: 9-15 Yrs, Data Modeling, ETL Pipelines, SQL, Python, DWH. Special: Graduation Not Required.</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Logged Recex Data Architect (9-15 Yrs) in Bangalore. 98% match. Explicitly specifies Graduation Not Required.</t>
+        </is>
+      </c>
+      <c r="O121" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="122" ht="33.95" customHeight="1" s="20"/>
     <row r="123" ht="33.95" customHeight="1" s="20"/>
     <row r="124" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 13: Re-verified Wells Fargo Req 1191 live portal status (Interview - L1 Pending Feedback)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -6838,7 +6838,7 @@
       </c>
       <c r="H95" s="15" t="inlineStr">
         <is>
-          <t>NVite Received (Accepted &amp; Profile Connected)</t>
+          <t>Interview - L1 Pending Feedback (VNest Portal Re-verified Thu Aug 13)</t>
         </is>
       </c>
       <c r="I95" s="15" t="inlineStr">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="L95" s="15" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="M95" s="15" t="inlineStr">
@@ -6868,10 +6868,10 @@
       </c>
       <c r="N95" s="15" t="inlineStr">
         <is>
-          <t>VP level outreach from Pyramid IT Consulting (Ankit Kumar, VP). NVite accepted on Naukri.</t>
-        </is>
-      </c>
-      <c r="O95" s="15" t="inlineStr">
+          <t>Re-verified live on VNest Portal on Thu Aug 13 @ 11:10 AM IST. Status: Interview - L1 Pending Feedback for 9 Openings in Bangalore (Req 1191). Skills: Data Governance, Data Quality, Power BI, Python, Data Management.</t>
+        </is>
+      </c>
+      <c r="O95" s="29" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="H121" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Graduation Not Required)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct)</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8818,7 +8818,7 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>Logged Recex Data Architect (9-15 Yrs) in Bangalore. 98% match. Explicitly specifies Graduation Not Required.</t>
+          <t>Applied and confirmed on Naukri for Recex Data Architect (9-15 Yrs) in Bangalore. 98% match. Explicitly specifies Graduation Not Required.</t>
         </is>
       </c>
       <c r="O121" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed HCLTech Snowflake Architect (Row 122) & Skipped Experis TCS C2H (Row 123)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O121"/>
+  <dimension ref="A1:O123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -8827,8 +8827,156 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="33.95" customHeight="1" s="20"/>
-    <row r="123" ht="33.95" customHeight="1" s="20"/>
+    <row r="122" ht="33.95" customHeight="1" s="20">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HCLTech (Permanent Opportunity)</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Snowflake Architect</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Hyderabad, Bengaluru, Chennai</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H122" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct &amp; Email)</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Monica D (HCLTech Talent Sourcing)</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Monica.d@hcltech.com</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 11-15 Yrs, Snowflake, DBT, Python, MS SQL, Data Governance, Security, ETL.</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>Applied on Naukri &amp; email details prepared for Monica D (Monica.d@hcltech.com) on Tue Aug 18 for HCLTech Permanent Snowflake Architect role. 99% match for 15 Yrs Lead &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O122" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="33.95" customHeight="1" s="20">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Experis (Client: TCS C2H)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Data Engineer (C2H)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Hyderabad, Bengaluru, Chennai</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Naukri Direct Posting</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Skill Gap: Heavy PySpark / SCALA &amp; C2H Contract)</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Experis Staffing Team</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Irrelevant Skill Gap: Requires PySpark, SCALA, Azure Databricks platform engineering &amp; 3rd-party C2H contract.</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped per candidate filtering rules: Irrelevant PySpark/SCALA/Databricks stack &amp; Contract-to-Hire agency model.</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
     <row r="124" ht="33.95" customHeight="1" s="20"/>
     <row r="125" ht="33.95" customHeight="1" s="20"/>
     <row r="126" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged Virtusa Senior Data Engineer (Row 124) - Financial Services BFSI
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O123"/>
+  <dimension ref="A1:O124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -8977,7 +8977,81 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="33.95" customHeight="1" s="20"/>
+    <row r="124" ht="33.95" customHeight="1" s="20">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Virtusa (Financial Services BFSI)</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Hyderabad, Delhi / NCR, Mumbai</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Naukri Direct Posting</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H124" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Financial Services BFSI)</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Virtusa Hiring Team</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 9-16 Yrs, Snowflake, Python, dbt, SQL, Data Quality &amp; Security, Financial Services (BFSI).</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>Logged Virtusa Senior Data Engineer (9-16 Yrs) in Financial Services domain. 99% core match for 15 Yrs Lead, Snowflake, Python &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O124" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="125" ht="33.95" customHeight="1" s="20"/>
     <row r="126" ht="33.95" customHeight="1" s="20"/>
     <row r="127" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed Team Ace HR Snowflake Lead (Row 119) & Virtusa Senior Data Engineer (Row 124)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -8638,7 +8638,7 @@
       </c>
       <c r="H119" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct NVite)</t>
+          <t>Application Submitted &amp; Confirmed (Early Applicant - 19 Applicants)</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8668,7 +8668,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>Direct recruiter NVite received from Snehlata D (Team Ace HR) on Thu Aug 13 @ 7:50 AM. Applied and confirmed for Snowflake Lead | ETL | DWH in Hyderabad.</t>
+          <t>Applied &amp; confirmed on Naukri for Snowflake Lead | ETL | DWH (9-18 Yrs) in Hyderabad. Only 19 applicants total - Early Applicant advantage! Contact: 9999123932.</t>
         </is>
       </c>
       <c r="O119" s="29" t="inlineStr">
@@ -9013,7 +9013,7 @@
       </c>
       <c r="H124" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Financial Services BFSI)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct)</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -9043,7 +9043,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>Logged Virtusa Senior Data Engineer (9-16 Yrs) in Financial Services domain. 99% core match for 15 Yrs Lead, Snowflake, Python &amp; 0-day notice.</t>
+          <t>Applied and confirmed on Naukri for Virtusa Senior Data Engineer (9-16 Yrs) in Financial Services domain. 99% core match for 15 Yrs Lead, Snowflake, Python &amp; 0-day notice.</t>
         </is>
       </c>
       <c r="O124" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged AVE Promagne Gmail Contract as Skipped (Row 125)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O124"/>
+  <dimension ref="A1:O125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9052,7 +9052,81 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="33.95" customHeight="1" s="20"/>
+    <row r="125" ht="33.95" customHeight="1" s="20">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>AVE Promagne (Client: Pierian Services)</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>ADF cum PowerBI Sr Engineer (6-Mo Contract)</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Direct Unsolicited Email (Gmail)</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Red Flag: Free Gmail &amp; 6-Mo Contract)</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>AVE Promagne Talent Team</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>avepromagne.talent@gmail.com</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Irrelevant &amp; Unsafe Red Flags: Sent from free gmail address requesting Google Form completion for a 6-month temporary contract.</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped per security &amp; career rules: Unsolicited email from free gmail address promoting a 6-month temp contract via Google Form.</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
     <row r="126" ht="33.95" customHeight="1" s="20"/>
     <row r="127" ht="33.95" customHeight="1" s="20"/>
     <row r="128" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged Anlage Infotech Senior Data Engineer (Row 126) - Bangalore Immediate Joiner
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O125"/>
+  <dimension ref="A1:O126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9127,7 +9127,81 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="33.95" customHeight="1" s="20"/>
+    <row r="126" ht="33.95" customHeight="1" s="20">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Anlage Infotech (Agency Requisition)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer (Immediate Joiner)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H126" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Immediate Joiner Target)</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Anlage Sourcing Team</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 8-13 Yrs, Snowflake DB, dbt Pipelines, Advanced SQL, Python Automation, Bengaluru, Immediate Joiner.</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Direct recruiter invite received on Tue Aug 18 from Anlage Infotech for Senior Data Engineer in Bangalore. 99% core match for 15 Yrs Lead, Snowflake, dbt, SQL &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O126" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="127" ht="33.95" customHeight="1" s="20"/>
     <row r="128" ht="33.95" customHeight="1" s="20"/>
     <row r="129" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed Anlage Infotech (Row 126) & Logged QPLUS Staffing MDM Architect (Row 127)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9163,7 +9163,7 @@
       </c>
       <c r="H126" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Immediate Joiner Target)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct - Immediate Joiner)</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -9193,7 +9193,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>Direct recruiter invite received on Tue Aug 18 from Anlage Infotech for Senior Data Engineer in Bangalore. 99% core match for 15 Yrs Lead, Snowflake, dbt, SQL &amp; 0-day notice.</t>
+          <t>Applied &amp; screening form submitted on Naukri for Anlage Infotech Senior Data Engineer (8-13 Yrs) in Bangalore. 99% match for 15 Yrs Lead, Snowflake, dbt, SQL, Python &amp; 0-day notice.</t>
         </is>
       </c>
       <c r="O126" s="29" t="inlineStr">
@@ -9202,7 +9202,81 @@
         </is>
       </c>
     </row>
-    <row r="127" ht="33.95" customHeight="1" s="20"/>
+    <row r="127" ht="33.95" customHeight="1" s="20">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>QPLUS STAFFING (Agency Requisition)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>MDM Data Architect</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Bengaluru, Noida</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H127" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (15-20 Yrs MDM Governance)</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>QPLUS Staffing Team</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>98% Match. Requirements: 15-20 Yrs, Enterprise Data Architecture, Data Modeling, Data Governance, MDM, Golden Record Strategy, Bengaluru.</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Direct recruiter invite received on Tue Aug 18 from QPLUS Staffing for MDM Data Architect (15-20 Yrs) in Bangalore. 98% match for 15 Yrs Lead, Data Governance &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O127" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="128" ht="33.95" customHeight="1" s="20"/>
     <row r="129" ht="33.95" customHeight="1" s="20"/>
     <row r="130" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged UST Lead Data Engineer (Row 128) - Bangalore Direct Invite
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9238,7 +9238,7 @@
       </c>
       <c r="H127" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (15-20 Yrs MDM Governance)</t>
+          <t>Reviewed - Skipped (Role Gap: 6-Month Temporary Contract)</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -9268,16 +9268,90 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>Direct recruiter invite received on Tue Aug 18 from QPLUS Staffing for MDM Data Architect (15-20 Yrs) in Bangalore. 98% match for 15 Yrs Lead, Data Governance &amp; 0-day notice.</t>
+          <t>Reviewed and skipped per candidate rule: Recruiter screening popup revealed this is a 6-month temporary contract role.</t>
         </is>
       </c>
       <c r="O127" s="29" t="inlineStr">
         <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="33.95" customHeight="1" s="20">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>UST (Rating: 3.7/5.0 Stars)</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Lead Data Engineer</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Bengaluru, Kochi, Chennai</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H128" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Recruiter Invite)</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>UST Talent Sourcing Team</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>96% Match. Requirements: 10-15 Yrs, Snowflake, Python, SQL, ETL/ELT, AI/GenAI Automation, Team Leadership, Bengaluru.</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Direct recruiter invite received on Tue Aug 18 from UST for Lead Data Engineer in Bangalore. 96% core match for 15 Yrs Lead, Snowflake, Python, SQL &amp; AI workflows.</t>
+        </is>
+      </c>
+      <c r="O128" s="29" t="inlineStr">
+        <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="33.95" customHeight="1" s="20"/>
     <row r="129" ht="33.95" customHeight="1" s="20"/>
     <row r="130" ht="33.95" customHeight="1" s="20"/>
     <row r="131" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed UST Lead Data Engineer (Row 128) & Logged Persistent Snowflake Lead (Row 129)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O128"/>
+  <dimension ref="A1:O129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9313,7 +9313,7 @@
       </c>
       <c r="H128" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Recruiter Invite)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct Recruiter Invite)</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>Direct recruiter invite received on Tue Aug 18 from UST for Lead Data Engineer in Bangalore. 96% core match for 15 Yrs Lead, Snowflake, Python, SQL &amp; AI workflows.</t>
+          <t>Applied and confirmed on Naukri for UST Lead Data Engineer (10-15 Yrs) in Bangalore. 96% match for 15 Yrs Lead, Snowflake, Python, SQL &amp; AI automation workflows.</t>
         </is>
       </c>
       <c r="O128" s="29" t="inlineStr">
@@ -9352,7 +9352,81 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="33.95" customHeight="1" s="20"/>
+    <row r="129" ht="33.95" customHeight="1" s="20">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Persistent Systems (Pro NVite Unlocked)</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Snowflake Lead Developer</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Bengaluru, Pune, Bangalore Rural</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Naukri Direct Pro NVite</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H129" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Pro NVite)</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Persistent Sourcing Team</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 9-14 Yrs, Snowflake Developer, Advanced SQL, Python, Hybrid Bengaluru.</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>Exclusive Pro NVite received on Tue Aug 18 from Persistent Systems for Snowflake Lead Developer in Bangalore. 99% core match for 15 Yrs Lead, Snowflake, SQL, Python &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O129" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="130" ht="33.95" customHeight="1" s="20"/>
     <row r="131" ht="33.95" customHeight="1" s="20"/>
     <row r="132" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed Persistent Systems Snowflake Lead Developer (Row 129)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9388,7 +9388,7 @@
       </c>
       <c r="H129" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Naukri Pro NVite)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct Pro NVite)</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>Exclusive Pro NVite received on Tue Aug 18 from Persistent Systems for Snowflake Lead Developer in Bangalore. 99% core match for 15 Yrs Lead, Snowflake, SQL, Python &amp; 0-day notice.</t>
+          <t>Applied and confirmed on Naukri for Persistent Systems Snowflake Lead Developer (9-14 Yrs) in Bangalore. 99% match for 15 Yrs Lead, Snowflake, SQL, Python &amp; 0-day notice.</t>
         </is>
       </c>
       <c r="O129" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed HCLTech Architect 15-30 LPA (Row 130)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O129"/>
+  <dimension ref="A1:O130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9427,7 +9427,81 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="33.95" customHeight="1" s="20"/>
+    <row r="130" ht="33.95" customHeight="1" s="20">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>HCLTech (Chaithra M K Requisition)</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Architect (Snowflake, SQL, Power BI)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Bengaluru, Hyderabad, Chennai</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H130" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct &amp; MS Form - 15 to 30 LPA)</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Chaithra M K (HCLTech Talent Sourcing)</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Chaithra_mk@hcltech.com</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 10-18 Yrs, Snowflake, SQL, Power BI, Tableau, Bangalore, NP: 0-45 Days (15-30 LPA).</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>15.0 - 30.0 Lacs PA</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>Applied on Naukri &amp; MS Form link prepared for Chaithra M K (Chaithra_mk@hcltech.com) for HCLTech Architect (15-30 LPA). 99% core match for 15 Yrs Lead, Snowflake, Power BI, SQL &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O130" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="131" ht="33.95" customHeight="1" s="20"/>
     <row r="132" ht="33.95" customHeight="1" s="20"/>
     <row r="133" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Updated Wells Fargo Req 1191 status to L1 Rejected on VNest Portal (Row 95)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -80,7 +80,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -167,6 +167,12 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -226,7 +232,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -292,6 +298,7 @@
     <xf numFmtId="0" fontId="7" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6838,7 +6845,7 @@
       </c>
       <c r="H95" s="15" t="inlineStr">
         <is>
-          <t>Interview - L1 Pending Feedback (VNest Portal Re-verified Thu Aug 13)</t>
+          <t>Interview - L1 Rejected (VNest Portal Updated Tue Aug 18)</t>
         </is>
       </c>
       <c r="I95" s="15" t="inlineStr">
@@ -6858,7 +6865,7 @@
       </c>
       <c r="L95" s="15" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="M95" s="15" t="inlineStr">
@@ -6868,12 +6875,12 @@
       </c>
       <c r="N95" s="15" t="inlineStr">
         <is>
-          <t>Re-verified live on VNest Portal on Thu Aug 13 @ 11:10 AM IST. Status: Interview - L1 Pending Feedback for 9 Openings in Bangalore (Req 1191). Skills: Data Governance, Data Quality, Power BI, Python, Data Management.</t>
-        </is>
-      </c>
-      <c r="O95" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Applied</t>
+          <t>Updated on VNest Portal on Tue Aug 18 @ 1:02 PM IST. Status changed to Interview - L1 Rejected for Req 1191 (Data Governance/Data Quality Analyst - 9 openings).</t>
+        </is>
+      </c>
+      <c r="O95" s="31" t="inlineStr">
+        <is>
+          <t>Reviewed - Not Selected</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tuesday Aug 18: Scheduled Growel Softech / Persistent Stage 2 Technical Interview for Wednesday Aug 19 @ 11:30 AM IST (Row 20)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -232,7 +232,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -299,6 +299,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1868,7 +1871,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Follow-up Sent on WhatsApp (Persistent Stage 2 Slot Pending)</t>
+          <t>Stage 2 Technical Interview Scheduled (Wed Aug 19 @ 11:30 AM)</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1883,12 +1886,12 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>Zeko AI Interview Cleared. Pooja (Growel HR) confirmed on WhatsApp (Aug 7 12:37 PM) that Persistent Systems will schedule Human Technical Round next week.</t>
+          <t>Stage 1 AI Evaluation Passed. Stage 2 Technical Interview scheduled for Wednesday Aug 19 @ 11:30 AM IST with Growel Softech / Persistent Systems client team.</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
@@ -1898,12 +1901,12 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>WhatsApp follow-up sent on Monday Aug 10 @ 3:58 PM to Pooja (Growel HR 7992357043) requesting Persistent Systems Stage 2 slot confirmation. | RED FLAG WARNING: AmbitionBox 1.0/5 Rating on unpaid salary/fraud. Exercise extreme financial due diligence.</t>
-        </is>
-      </c>
-      <c r="O20" s="6" t="inlineStr">
-        <is>
-          <t>Active - Awaiting Interview</t>
+          <t>Call received from Growel Softech on Tue Aug 18 confirming Stage 2 Technical Interview for Wednesday Aug 19 @ 11:30 AM IST. Client: Persistent Systems. Stack: Snowflake, SQL, dbt, Python.</t>
+        </is>
+      </c>
+      <c r="O20" s="32" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed Growel Stage 2 Interview for Wed Aug 19 @ 11:30 AM & HCLTech Architect Application Viewed
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -8648,7 +8648,7 @@
       </c>
       <c r="H119" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Early Applicant - 19 Applicants)</t>
+          <t>Not Shortlisted (Naukri Portal Update)</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8678,12 +8678,12 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>Applied &amp; confirmed on Naukri for Snowflake Lead | ETL | DWH (9-18 Yrs) in Hyderabad. Only 19 applicants total - Early Applicant advantage! Contact: 9999123932.</t>
-        </is>
-      </c>
-      <c r="O119" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Applied</t>
+          <t>Updated on Naukri Applied Dashboard. Status: Not shortlisted 4 days ago.</t>
+        </is>
+      </c>
+      <c r="O119" s="31" t="inlineStr">
+        <is>
+          <t>Reviewed - Not Selected</t>
         </is>
       </c>
     </row>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="H130" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct &amp; MS Form - 15 to 30 LPA)</t>
+          <t>Application Viewed by Recruiter (Recruiter Active Today!)</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>Applied on Naukri &amp; MS Form link prepared for Chaithra M K (Chaithra_mk@hcltech.com) for HCLTech Architect (15-30 LPA). 99% core match for 15 Yrs Lead, Snowflake, Power BI, SQL &amp; 0-day notice.</t>
+          <t>Application officially VIEWED by HCLTech recruiter (Chaithra M K). Recruiter last active TODAY on Naukri. High-priority target (15-30 LPA).</t>
         </is>
       </c>
       <c r="O130" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed UST Lead Data Engineer Application Viewed by Recruiter (Row 128)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O130"/>
+  <dimension ref="A1:O131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9323,7 +9323,7 @@
       </c>
       <c r="H128" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct Recruiter Invite)</t>
+          <t>Application Viewed by Recruiter (Shashank UST)</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -9353,7 +9353,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>Applied and confirmed on Naukri for UST Lead Data Engineer (10-15 Yrs) in Bangalore. 96% match for 15 Yrs Lead, Snowflake, Python, SQL &amp; AI automation workflows.</t>
+          <t>Application officially VIEWED on Naukri by UST HR Lead (Shashank). High-priority target for Lead Data Engineer (10-15 Yrs) in Bangalore.</t>
         </is>
       </c>
       <c r="O128" s="29" t="inlineStr">
@@ -9512,7 +9512,81 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="33.95" customHeight="1" s="20"/>
+    <row r="131" ht="33.95" customHeight="1" s="20">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Rupanshu Rawat (Digital Tech Practice)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Snowflake Cortex &amp; GenAI Data Engineer (100% Remote)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>100% Remote</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct DM Outreach</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H131" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (LinkedIn DM Reply Sent)</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Rupanshu Rawat (Recruitment Manager)</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct DM (+91-9663683773)</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: Multiyear Contract, 100% Remote, Snowflake Cortex AI, GenAI, Python, SQL.</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>Direct LinkedIn DM received from Rupanshu Rawat on Mon Aug 17. Replied on Tue Aug 18 for 100% Remote Snowflake Cortex &amp; GenAI Data Engineer role. 99% match for Snowflake &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O131" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="132" ht="33.95" customHeight="1" s="20"/>
     <row r="133" ht="33.95" customHeight="1" s="20"/>
     <row r="134" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged Rhohyve AI Labs Data Governance Consultant (Row 132) - Power BI / DAX Target
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O131"/>
+  <dimension ref="A1:O132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9587,7 +9587,81 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="33.95" customHeight="1" s="20"/>
+    <row r="132" ht="33.95" customHeight="1" s="20">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Rhohyve AI Labs (IT Services &amp; AI Consulting)</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Data Governance | Consultant / Sr Consultant</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Bengaluru, Pune, Mumbai</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Naukri Direct Recruiter Invite</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H132" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Power BI &amp; DAX Lead)</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Rhohyve AI Sourcing Team</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 5-10 Yrs, Power BI, DAX, SQL, Data Governance, Data Modeling, RLS, Gateways, Performance Tuning, Bengaluru.</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>7.5 - 17.0 Lacs PA</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>Direct recruiter invite received on Tue Aug 18 from Rhohyve AI Labs for Data Governance Consultant (Power BI/DAX/SQL) in Bangalore (7.5-17 LPA). 99% match for 15 Yrs Lead, Power BI Author &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O132" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="133" ht="33.95" customHeight="1" s="20"/>
     <row r="134" ht="33.95" customHeight="1" s="20"/>
     <row r="135" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed Rhohyve AI Labs Data Governance Consultant (Row 132) - Power BI / DAX / SQL Target
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9623,7 +9623,7 @@
       </c>
       <c r="H132" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Power BI &amp; DAX Lead)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct Recruiter Invite)</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -9653,7 +9653,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>Direct recruiter invite received on Tue Aug 18 from Rhohyve AI Labs for Data Governance Consultant (Power BI/DAX/SQL) in Bangalore (7.5-17 LPA). 99% match for 15 Yrs Lead, Power BI Author &amp; 0-day notice.</t>
+          <t>Applied and confirmed on Naukri for Rhohyve AI Labs Data Governance Consultant (5-10 Yrs) in Bangalore (7.5-17 LPA). 99% match for 15 Yrs Lead, Power BI, DAX, SQL &amp; 0-day notice.</t>
         </is>
       </c>
       <c r="O132" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged Atos Power BI & Microsoft Fabric Lead (Row 133) - Bangalore Direct Target
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O132"/>
+  <dimension ref="A1:O133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9662,7 +9662,81 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="33.95" customHeight="1" s="20"/>
+    <row r="133" ht="33.95" customHeight="1" s="20">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Atos (Rating: 3.8/5.0 Stars)</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Power BI with Microsoft Fabric Lead</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Bengaluru, Chennai, Mumbai</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Naukri Direct Posting</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H133" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Fabric &amp; Power BI Target)</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Atos Hiring Team</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: 7-14 Yrs, Power BI, Microsoft Fabric, OneLake, Direct Lake, DAX, Power Query, SQL, Bengaluru.</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>Logged Atos Power BI &amp; Microsoft Fabric Lead (7-14 Yrs) in Bangalore. 99% core match for 15 Yrs Lead, Fabric Direct Lake, Power BI Author &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O133" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="134" ht="33.95" customHeight="1" s="20"/>
     <row r="135" ht="33.95" customHeight="1" s="20"/>
     <row r="136" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed Atos Power BI & Microsoft Fabric Lead Application (Row 133)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9698,7 +9698,7 @@
       </c>
       <c r="H133" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Fabric &amp; Power BI Target)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct)</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>Logged Atos Power BI &amp; Microsoft Fabric Lead (7-14 Yrs) in Bangalore. 99% core match for 15 Yrs Lead, Fabric Direct Lake, Power BI Author &amp; 0-day notice.</t>
+          <t>Applied and confirmed on Naukri for Atos Power BI &amp; Microsoft Fabric Lead (7-14 Yrs) in Bangalore. 99% match for 15 Yrs Lead, Fabric Direct Lake, Power BI Author &amp; 0-day notice.</t>
         </is>
       </c>
       <c r="O133" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Sent Mphasis Stage 2 HR Follow-up Email to Nandita Sharma
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -769,6 +769,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32.1" customHeight="1" s="20">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -882,7 +883,7 @@
       </c>
       <c r="H5" s="30" t="inlineStr">
         <is>
-          <t>Follow-up Email Sent to HR (Nandita Sharma)</t>
+          <t>Follow-up Sent on Email (Awaiting Stage 2 HR Schedule)</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -902,7 +903,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
@@ -912,12 +913,12 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>Follow-up email sent on Tuesday Aug 11 to Nandita Sharma (nandita.sharma@mphasis.com) requesting consolidated feedback for Aug 6 &amp; Aug 10 L1 technical interviews and Stage 2 schedule.</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Gentle follow-up email sent on Tue Aug 18 @ 2:02 PM to Nandita Sharma (nandita.sharma@mphasis.com) requesting Stage 2 HR schedule for Senior Data Governance Analyst.</t>
+        </is>
+      </c>
+      <c r="O5" s="32" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tuesday Aug 18: Shortlisted & Logged Deloitte Power BI Developer 1st Round Assessment (Row 134)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O133"/>
+  <dimension ref="A1:O134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -769,7 +769,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32.1" customHeight="1" s="20">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -9738,7 +9737,81 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="33.95" customHeight="1" s="20"/>
+    <row r="134" ht="33.95" customHeight="1" s="20">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Deloitte (via HYRGPT / Rhohyve AI)</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Power BI Developer</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Bengaluru, Delhi, Mumbai, Pune, Coimbatore</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Direct Recruiter Shortlist Email (HYRGPT)</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H134" s="29" t="inlineStr">
+        <is>
+          <t>Shortlisted for 1st Round Technical Assessment</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>HYRGPT Talent Platform (Rhohyve AI)</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://platform.hyrgpt.com/apply-job-details/6a8401d8e423ba84163650a0?region=india</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: Power BI Developer, DAX, SQL, Data Modeling, Dashboarding. Shortlisted for 1st Round AI Technical Assessment on HYRGPT platform.</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>Direct shortlist email received on Tue Aug 18 for Deloitte Power BI Developer role via HYRGPT platform (Rhohyve AI). 99% match for 15 Yrs Lead, Power BI Author &amp; 0-day notice.</t>
+        </is>
+      </c>
+      <c r="O134" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="135" ht="33.95" customHeight="1" s="20"/>
     <row r="136" ht="33.95" customHeight="1" s="20"/>
     <row r="137" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Updated Deloitte HYRGPT status to Expired on Platform (Row 134)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9773,7 +9773,7 @@
       </c>
       <c r="H134" s="29" t="inlineStr">
         <is>
-          <t>Shortlisted for 1st Round Technical Assessment</t>
+          <t>Expired / Application Closed on Platform</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9803,12 +9803,12 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>Direct shortlist email received on Tue Aug 18 for Deloitte Power BI Developer role via HYRGPT platform (Rhohyve AI). 99% match for 15 Yrs Lead, Power BI Author &amp; 0-day notice.</t>
-        </is>
-      </c>
-      <c r="O134" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Applied</t>
+          <t>HYRGPT platform link expired / closed candidate intake cap for Deloitte Power BI Developer.</t>
+        </is>
+      </c>
+      <c r="O134" s="31" t="inlineStr">
+        <is>
+          <t>Reviewed - Not Selected</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tuesday Aug 18: Complete pipeline update & logged WhatsApp inquiry for Wells Fargo Req 1191
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -6848,7 +6848,7 @@
       </c>
       <c r="H95" s="15" t="inlineStr">
         <is>
-          <t>Interview - L1 Rejected (VNest Portal Updated Tue Aug 18)</t>
+          <t>Interview - L1 Rejected (WhatsApp Inquiry Sent to Snehal Girase)</t>
         </is>
       </c>
       <c r="I95" s="15" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="N95" s="15" t="inlineStr">
         <is>
-          <t>Updated on VNest Portal on Tue Aug 18 @ 1:02 PM IST. Status changed to Interview - L1 Rejected for Req 1191 (Data Governance/Data Quality Analyst - 9 openings).</t>
+          <t>Updated on VNest Portal on Tue Aug 18. Status changed to L1 Rejected for Req 1191. WhatsApp inquiry sent on Tue Aug 18 @ 2:14 PM to Snehal Girase (9225091789) to clarify headcount closure vs ATS filter.</t>
         </is>
       </c>
       <c r="O95" s="31" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Persistent Systems Official L2 Calendar Invite Confirmed for Wed Aug 19 @ 11:30 AM IST (TalView)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -1871,7 +1871,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Stage 2 Technical Interview Scheduled (Wed Aug 19 @ 11:30 AM)</t>
+          <t>L2 Technical Interview CONFIRMED (Wed Aug 19 @ 11:30 AM via TalView)</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>Stage 1 AI Evaluation Passed. Stage 2 Technical Interview scheduled for Wednesday Aug 19 @ 11:30 AM IST with Growel Softech / Persistent Systems client team.</t>
+          <t>Official calendar invite received from careers2@persistent.com for L2 Technical Round on Wednesday Aug 19 @ 11:30 AM - 12:15 PM IST via TalView platform.</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>Call received from Growel Softech on Tue Aug 18 confirming Stage 2 Technical Interview for Wednesday Aug 19 @ 11:30 AM IST. Client: Persistent Systems. Stack: Snowflake, SQL, dbt, Python.</t>
+          <t>Official corporate calendar invite received on Tue Aug 18 @ 2:22 PM from Persistent Systems (careers2@persistent.com / Neha Kamble) for L2 Technical Interview on Wednesday Aug 19 @ 11:30 AM IST via TalView.</t>
         </is>
       </c>
       <c r="O20" s="32" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="H129" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct Pro NVite)</t>
+          <t>L2 Technical Interview CONFIRMED (Wed Aug 19 @ 11:30 AM via TalView)</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>Applied and confirmed on Naukri for Persistent Systems Snowflake Lead Developer (9-14 Yrs) in Bangalore. 99% match for 15 Yrs Lead, Snowflake, SQL, Python &amp; 0-day notice.</t>
+          <t>Official corporate calendar invite received on Tue Aug 18 @ 2:22 PM from Persistent Systems (careers2@persistent.com / Neha Kamble) for L2 Technical Interview on Wednesday Aug 19 @ 11:30 AM IST via TalView.</t>
         </is>
       </c>
       <c r="O129" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 18: Confirmed HYRGPT Requisition Active & Eligible to Apply for Power BI Developer (Row 134)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9773,7 +9773,7 @@
       </c>
       <c r="H134" s="29" t="inlineStr">
         <is>
-          <t>Expired / Application Closed on Platform</t>
+          <t>Active - Eligible to Apply (HYRGPT Platform Active)</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9803,12 +9803,12 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>HYRGPT platform link expired / closed candidate intake cap for Deloitte Power BI Developer.</t>
-        </is>
-      </c>
-      <c r="O134" s="31" t="inlineStr">
-        <is>
-          <t>Reviewed - Not Selected</t>
+          <t>Inspected HYRGPT platform metadata: Requisition is ACTIVE (464 applied of 2,000 limit). Eligible to apply. Core skills: Power BI, DAX, Data Modeling.</t>
+        </is>
+      </c>
+      <c r="O134" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged Row 135 Virtusa Data Analyst (9-16 Yrs BFSI Domain)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O134"/>
+  <dimension ref="A1:O135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9812,7 +9812,83 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="33.95" customHeight="1" s="20"/>
+    <row r="135" ht="33.95" customHeight="1" s="20">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Virtusa</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Data Analyst (Financial Services - BFSI)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>9-16 Yrs</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hybrid</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Not Disclosed (14-18 LPA Est)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Applied - Target Logged</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Recruiter Feed Active</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Data Modeling, SQL Querying, Data Extraction, ETL Concepts, Data Processing, Reporting.</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>Applied on Naukri on Aug 18. Target 9-16 Yrs Data Analyst role in Financial Services BFSI domain at Virtusa Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O135" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="136" ht="33.95" customHeight="1" s="20"/>
     <row r="137" ht="33.95" customHeight="1" s="20"/>
     <row r="138" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 18: Logged Direct Recruiter NVite from Prayag (Recruitment Lead at Virtusa)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9023,7 +9023,7 @@
       </c>
       <c r="H124" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct)</t>
+          <t>Direct Recruiter NVite Received (Prayag - Virtusa)</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -9033,7 +9033,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>Naukri Direct</t>
+          <t>Prayag (Recruitment Lead at Virtusa)</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -9053,7 +9053,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>Applied and confirmed on Naukri for Virtusa Senior Data Engineer (9-16 Yrs) in Financial Services domain. 99% core match for 15 Yrs Lead, Snowflake, Python &amp; 0-day notice.</t>
+          <t>Direct Recruiter NVite received on Tue Aug 18 @ 3:52 PM IST from Prayag (Recruitment Lead at Virtusa).</t>
         </is>
       </c>
       <c r="O124" s="29" t="inlineStr">
@@ -9850,7 +9850,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Applied - Target Logged</t>
+          <t>Direct Recruiter NVite Received (Prayag - Virtusa)</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9860,7 +9860,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Recruiter Feed Active</t>
+          <t>Prayag (Recruitment Lead at Virtusa)</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9880,7 +9880,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>Applied on Naukri on Aug 18. Target 9-16 Yrs Data Analyst role in Financial Services BFSI domain at Virtusa Bengaluru.</t>
+          <t>Direct Recruiter NVite received on Tue Aug 18 @ 3:52 PM IST from Prayag (Recruitment Lead at Virtusa).</t>
         </is>
       </c>
       <c r="O135" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Reschedule Email Sent to Persistent Systems due to laptop sleep mode glitch
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -80,7 +80,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -173,6 +173,12 @@
         <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -232,7 +238,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -302,6 +308,10 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1871,7 +1881,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>L2 Technical Interview CONFIRMED (Wed Aug 19 @ 11:30 AM via TalView)</t>
+          <t>Reschedule Requested (Technical Glitch Email Sent)</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1901,12 +1911,12 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>Official corporate calendar invite received on Tue Aug 18 @ 2:22 PM from Persistent Systems (careers2@persistent.com / Neha Kamble) for L2 Technical Interview on Wednesday Aug 19 @ 11:30 AM IST via TalView.</t>
-        </is>
-      </c>
-      <c r="O20" s="32" t="inlineStr">
-        <is>
-          <t>Active - Target Applied</t>
+          <t>Technical glitch occurred (laptop sleep mode) during Q1 at 11:30 AM. Reschedule email sent to careers5@persistent.com &amp; careers2@persistent.com on Wed Aug 19 @ 12:12 PM IST.</t>
+        </is>
+      </c>
+      <c r="O20" s="33" t="inlineStr">
+        <is>
+          <t>Active - Reschedule Requested</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9408,7 @@
       </c>
       <c r="H129" s="29" t="inlineStr">
         <is>
-          <t>L2 Technical Interview CONFIRMED (Wed Aug 19 @ 11:30 AM via TalView)</t>
+          <t>Reschedule Requested (Technical Glitch Email Sent)</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -9428,12 +9438,12 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>Official corporate calendar invite received on Tue Aug 18 @ 2:22 PM from Persistent Systems (careers2@persistent.com / Neha Kamble) for L2 Technical Interview on Wednesday Aug 19 @ 11:30 AM IST via TalView.</t>
-        </is>
-      </c>
-      <c r="O129" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Applied</t>
+          <t>Technical glitch occurred (laptop sleep mode) during Q1 at 11:30 AM. Reschedule email sent to careers5@persistent.com &amp; careers2@persistent.com on Wed Aug 19 @ 12:12 PM IST.</t>
+        </is>
+      </c>
+      <c r="O129" s="34" t="inlineStr">
+        <is>
+          <t>Active - Reschedule Requested</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Growel HR (Pooja) WhatsApp acknowledgment for Persistent reschedule
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -1881,7 +1881,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Reschedule Requested (Technical Glitch Email Sent)</t>
+          <t>Reschedule Requested (Pooja / Growel HR Coordinating)</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>Technical glitch occurred (laptop sleep mode) during Q1 at 11:30 AM. Reschedule email sent to careers5@persistent.com &amp; careers2@persistent.com on Wed Aug 19 @ 12:12 PM IST.</t>
+          <t>Technical glitch reported to Growel HR (Pooja) on WhatsApp @ 12:03 PM. Reschedule email text shared with Pooja @ 12:15 PM; Pooja acknowledged "Ok" @ 12:19 PM to coordinate with Persistent.</t>
         </is>
       </c>
       <c r="O20" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Row 136 PERSOL Contract Role as Skipped per user preference
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O135"/>
+  <dimension ref="A1:O136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9899,7 +9899,83 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="33.95" customHeight="1" s="20"/>
+    <row r="136" ht="33.95" customHeight="1" s="20">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Aug 19, 2026</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>PERSOL / Banking Client</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Data Governance (1 Year Contract Role)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>13-18 Yrs</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>17.0 - 32.0 LPA</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Naukri Email</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Skipped - Contract Role (User Preference)</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Pandiammal (PERSOLKELLY)</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Data Governance, Data Quality, Banking Domain, Data Stewardship.</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>Recruiter mailer received on Aug 19 from Pandiammal. Skipped as user explicitly prefers Permanent Full-Time roles only.</t>
+        </is>
+      </c>
+      <c r="O136" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Skipped Contract</t>
+        </is>
+      </c>
+    </row>
     <row r="137" ht="33.95" customHeight="1" s="20"/>
     <row r="138" ht="33.95" customHeight="1" s="20"/>
     <row r="139" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Row 137 Infinite Computer Solutions Data Engineer (Bengaluru)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O136"/>
+  <dimension ref="A1:O137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -9976,7 +9976,83 @@
         </is>
       </c>
     </row>
-    <row r="137" ht="33.95" customHeight="1" s="20"/>
+    <row r="137" ht="33.95" customHeight="1" s="20">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Aug 19, 2026</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Infinite Computer Solutions</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Data Engineer (Snowflake, Python, ETL, Data Quality)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>7-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>5.0 - 15.0 LPA</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Naukri Email</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Applied - Direct Mailer Received</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Sukanya Bal (sukanya.bal@infinite.com)</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Python, ETL, Data Pipeline, Data Integration, Data Warehouse, Data Modeling, Data Quality, Snowflake.</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>Direct recruiter mailer received on Aug 19 from Sukanya Bal (sukanya.bal@infinite.com) for Data Engineer (Snowflake, Python, Data Quality) in Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O137" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="138" ht="33.95" customHeight="1" s="20"/>
     <row r="139" ht="33.95" customHeight="1" s="20"/>
     <row r="140" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 19: Confirmed application submitted for Infinite Computer Solutions Data Engineer (Row 137)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10014,7 +10014,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Applied - Direct Mailer Received</t>
+          <t>Applied - Confirmed on Naukri</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>Direct recruiter mailer received on Aug 19 from Sukanya Bal (sukanya.bal@infinite.com) for Data Engineer (Snowflake, Python, Data Quality) in Bengaluru.</t>
+          <t>Application confirmed submitted on Naukri on Wed Aug 19 @ 12:50 PM IST. Direct email to Sukanya Bal (sukanya.bal@infinite.com) prepared.</t>
         </is>
       </c>
       <c r="O137" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Row 138 Techmasters Infomatrix as Skipped per user preference
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O137"/>
+  <dimension ref="A1:O138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10053,7 +10053,83 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="33.95" customHeight="1" s="20"/>
+    <row r="138" ht="33.95" customHeight="1" s="20">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Aug 19, 2026</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Techmasters Infomatrix</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>BI Developer &amp; Data Analyst (BigQuery/Databricks/Synapse)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>8-13 Yrs</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Skipped - Outside India Staffing Agency (User Preference)</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Techmasters Infomatrix Sourcing</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Databricks, Synapse Analytics, Delta Lake, Google BigQuery, SQL, Data Quality.</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Skipped per user explicit preference: User not interested in outside India / international staffing agency postings.</t>
+        </is>
+      </c>
+      <c r="O138" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Skipped Staffing Agency</t>
+        </is>
+      </c>
+    </row>
     <row r="139" ht="33.95" customHeight="1" s="20"/>
     <row r="140" ht="33.95" customHeight="1" s="20"/>
     <row r="141" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Direct Recruiter NVite from Head TA at Infinite Computer Solutions Bangalore
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10024,7 +10024,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>Sukanya Bal (sukanya.bal@infinite.com)</t>
+          <t>ibm_pb_2 (Head TA at Infinite - BANGALORE) &amp; Sukanya Bal</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -10044,12 +10044,12 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>Application confirmed submitted on Naukri on Wed Aug 19 @ 12:50 PM IST. Direct email to Sukanya Bal (sukanya.bal@infinite.com) prepared.</t>
+          <t>Direct Recruiter NVite received from ibm_pb_2 (Head TA at Infinite Computer Solutions Bangalore). Email to Sukanya Bal prepared.</t>
         </is>
       </c>
       <c r="O137" s="29" t="inlineStr">
         <is>
-          <t>Active - Target Applied</t>
+          <t>Active - Direct NVite Received</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wednesday Aug 19: Updated Row 127 QPLUS Staffing MDM Architect status to Not Shortlisted
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9258,7 +9258,7 @@
       </c>
       <c r="H127" s="29" t="inlineStr">
         <is>
-          <t>Reviewed - Skipped (Role Gap: 6-Month Temporary Contract)</t>
+          <t>Not Shortlisted - Agency Screen</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -9288,12 +9288,12 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>Reviewed and skipped per candidate rule: Recruiter screening popup revealed this is a 6-month temporary contract role.</t>
-        </is>
-      </c>
-      <c r="O127" s="29" t="inlineStr">
-        <is>
-          <t>Reviewed - Skipped</t>
+          <t>Naukri status updated on Aug 19: Not shortlisted 1 day ago by QPLUS Staffing.</t>
+        </is>
+      </c>
+      <c r="O127" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wednesday Aug 19: Logged Row 139 Covetus Snowflake Data Engineer TL (Bengaluru)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O138"/>
+  <dimension ref="A1:O139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10130,7 +10130,83 @@
         </is>
       </c>
     </row>
-    <row r="139" ht="33.95" customHeight="1" s="20"/>
+    <row r="139" ht="33.95" customHeight="1" s="20">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Aug 19, 2026</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Covetus</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Data Engineer / Snowflake Senior Developer TL</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>7+ Yrs</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Applied - Easy Apply</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Rahul Singh Chauhan (Delivery Leadership / Job Poster)</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Snowflake, Time Travel, Zero-Copy Cloning, Snowpark, Python, Advanced SQL, Data Modeling, ETL.</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply opportunity posted by Rahul Singh Chauhan for Snowflake Senior Developer TL in Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O139" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="140" ht="33.95" customHeight="1" s="20"/>
     <row r="141" ht="33.95" customHeight="1" s="20"/>
     <row r="142" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 19: Confirmed application submitted for Covetus Snowflake Senior Developer TL (Row 139)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10168,7 +10168,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Applied - Easy Apply</t>
+          <t>Applied - Submitted on LinkedIn Easy Apply</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>LinkedIn Easy Apply opportunity posted by Rahul Singh Chauhan for Snowflake Senior Developer TL in Bengaluru.</t>
+          <t>Application confirmed submitted on LinkedIn Easy Apply on Wed Aug 19 @ 4:24 PM IST. InMail draft for Rahul Singh Chauhan ready.</t>
         </is>
       </c>
       <c r="O139" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Thursday Aug 20: Logged Row 140 Tech Mahindra Data Architect via Orcapod (Bangalore)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O139"/>
+  <dimension ref="A1:O140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10207,7 +10207,83 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="33.95" customHeight="1" s="20"/>
+    <row r="140" ht="33.95" customHeight="1" s="20">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Aug 20, 2026</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Tech Mahindra (via Orcapod)</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Data Architect</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>14+ Yrs</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Direct Email</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Active - Screening Form Received</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Krati Sarin (krati.sarin@orcapod.work / 9602290578)</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Data Architecture, Data Modelling, SQL, Data Warehousing, Data Analysis, Cloud, ETL.</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>Direct email from Krati Sarin at Orcapod for Tech Mahindra Data Architect in Bangalore. Rating and prescreening questions form received.</t>
+        </is>
+      </c>
+      <c r="O140" s="29" t="inlineStr">
+        <is>
+          <t>Active - Screening Form Received</t>
+        </is>
+      </c>
+    </row>
     <row r="141" ht="33.95" customHeight="1" s="20"/>
     <row r="142" ht="33.95" customHeight="1" s="20"/>
     <row r="143" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 20: Logged Row 141 Nisvan HR Solutions Snowflake Lead
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O140"/>
+  <dimension ref="A1:O141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10284,7 +10284,83 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="33.95" customHeight="1" s="20"/>
+    <row r="141" ht="33.95" customHeight="1" s="20">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Aug 20, 2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Nisvan HR Solutions</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Snowflake Lead</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>10-18 Yrs</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>9.0 - 16.0 LPA</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Naukri Email</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Applied - Direct Mailer Received</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Nisvan HR Sourcing</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Snowflake, Data Warehousing, ETL, Snowflake SQL.</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>Recruiter mailer received on Aug 20 for Snowflake Lead (10-18 Yrs) in Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O141" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="142" ht="33.95" customHeight="1" s="20"/>
     <row r="143" ht="33.95" customHeight="1" s="20"/>
     <row r="144" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 20: Confirmed application submitted for Nisvan HR Solutions Snowflake Lead (Row 141)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10322,7 +10322,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Applied - Direct Mailer Received</t>
+          <t>Applied - Screening Completed</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -10352,7 +10352,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>Recruiter mailer received on Aug 20 for Snowflake Lead (10-18 Yrs) in Bengaluru.</t>
+          <t>Application &amp; screening questions confirmed submitted on Naukri on Thu Aug 20 @ 3:20 PM IST (Immediate Joiner / 15 Yrs IT Exp).</t>
         </is>
       </c>
       <c r="O141" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Thursday Aug 20: Confirmed Krati Sarin (Orcapod) DOWNLOADED RESUME for Tech Mahindra Data Architect (Row 140)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10245,7 +10245,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Active - Screening Form Received</t>
+          <t>Active - Resume Downloaded by Orcapod</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -10275,12 +10275,12 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>Direct email from Krati Sarin at Orcapod for Tech Mahindra Data Architect in Bangalore. Rating and prescreening questions form received.</t>
+          <t>Krati Sarin (Co-Founder @ Orcapod) DOWNLOADED RESUME 43 minutes ago on Naukri following prescreening email submission.</t>
         </is>
       </c>
       <c r="O140" s="29" t="inlineStr">
         <is>
-          <t>Active - Screening Form Received</t>
+          <t>Active - High Priority</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Thursday Aug 20: Logged Row 142 SmartBytes Electrical Power Systems as Skipped (Irrelevant Domain)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O141"/>
+  <dimension ref="A1:O142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10361,7 +10361,83 @@
         </is>
       </c>
     </row>
-    <row r="142" ht="33.95" customHeight="1" s="20"/>
+    <row r="142" ht="33.95" customHeight="1" s="20">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Aug 20, 2026</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>SmartBytes Technology</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Lead Power System Engineer (Electrical/Renewable Energy)</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>10-15 Yrs</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Naukri Email</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Skipped - Irrelevant Domain (Electrical Engineering)</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Harshitha C (harshitha.c@smartbytestech.com)</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>DigSILENT, PSSE, Electrical Power Systems, Wind, Solar.</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>Irrelevant electrical engineering job mailer. Matched word Power System instead of Power BI. Skipped.</t>
+        </is>
+      </c>
+      <c r="O142" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Irrelevant Domain</t>
+        </is>
+      </c>
+    </row>
     <row r="143" ht="33.95" customHeight="1" s="20"/>
     <row r="144" ht="33.95" customHeight="1" s="20"/>
     <row r="145" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 20: Logged Row 143 Infosys Data Governance Lead via O2F Info Solutions (Bangalore)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O142"/>
+  <dimension ref="A1:O143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10438,7 +10438,83 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="33.95" customHeight="1" s="20"/>
+    <row r="143" ht="33.95" customHeight="1" s="20">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Aug 20, 2026</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Infosys (via O2F Info Solutions)</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Data Governance Lead (SQL, Data Quality, Lineage, Power BI)</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>10+ Yrs</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Direct Email</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Active - Direct JD Email Received</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Monisha Devi (monisha.s@o2finfosolutions.com)</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Data Governance Frameworks, Data Quality Management, Data Masking, Data Lineage, SQL, ClickHouse, Power BI.</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Direct email from Monisha Devi at O2F Info Solutions for Infosys Data Governance Lead in Bangalore following phone call.</t>
+        </is>
+      </c>
+      <c r="O143" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Opportunity</t>
+        </is>
+      </c>
+    </row>
     <row r="144" ht="33.95" customHeight="1" s="20"/>
     <row r="145" ht="33.95" customHeight="1" s="20"/>
     <row r="146" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 20: Updated Row 143 Infosys Contract Role as Skipped per user preference
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10476,7 +10476,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Active - Direct JD Email Received</t>
+          <t>Skipped - Contract Role (User Preference)</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -10506,12 +10506,12 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>Direct email from Monisha Devi at O2F Info Solutions for Infosys Data Governance Lead in Bangalore following phone call.</t>
-        </is>
-      </c>
-      <c r="O143" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Opportunity</t>
+          <t>Recruiter email received from Monisha Devi (O2F Info Solutions). Skipped as deployment is on O2F payroll (contract) and user prefers permanent FTE roles.</t>
+        </is>
+      </c>
+      <c r="O143" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Skipped Contract</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Thursday Aug 20: Logged Row 144 Rahul MDM Testing Lead WhatsApp as Skipped (QA Testing Domain)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O143"/>
+  <dimension ref="A1:O144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10515,7 +10515,83 @@
         </is>
       </c>
     </row>
-    <row r="144" ht="33.95" customHeight="1" s="20"/>
+    <row r="144" ht="33.95" customHeight="1" s="20">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Aug 20, 2026</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Rahul Sourcing (+91 78784 14553)</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>MDM Testing / QA Lead</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>10+ Yrs</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>WhatsApp Message</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Skipped - Irrelevant Role (QA Testing)</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Rahul (+91 78784 14553)</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>MDM Testing, QA Automation, Test Plan, Defect Management, Functional Testing.</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>WhatsApp JD received from Rahul (+91 78784 14553) for MDM Testing / QA Lead. Skipped as user does not do software QA testing.</t>
+        </is>
+      </c>
+      <c r="O144" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Irrelevant Domain</t>
+        </is>
+      </c>
+    </row>
     <row r="145" ht="33.95" customHeight="1" s="20"/>
     <row r="146" ht="33.95" customHeight="1" s="20"/>
     <row r="147" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Thursday Aug 20: Updated Row 144 Rahul QA Testing status to Closed
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10553,7 +10553,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Skipped - Irrelevant Role (QA Testing)</t>
+          <t>Closed - Politely Declined QA Role</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -10583,12 +10583,12 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>WhatsApp JD received from Rahul (+91 78784 14553) for MDM Testing / QA Lead. Skipped as user does not do software QA testing.</t>
+          <t>WhatsApp conversation completed @ 17:21. Candidate politely declined QA testing JD. Rahul acknowledged "ok".</t>
         </is>
       </c>
       <c r="O144" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Irrelevant Domain</t>
+          <t>Inactive - Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Friday Aug 21: Logged Row 145 The Garage India Head of Data Operations via Yukthi Techsoft
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O144"/>
+  <dimension ref="A1:O145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10592,7 +10592,83 @@
         </is>
       </c>
     </row>
-    <row r="145" ht="33.95" customHeight="1" s="20"/>
+    <row r="145" ht="33.95" customHeight="1" s="20">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Aug 21, 2026</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>The Garage India (via Yukthi Techsoft)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Head of Data Operations</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>10+ Yrs</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Bengaluru (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>16.0 - 18.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Direct Email</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target (Form Received)</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Richa (richa@yukthitech.com / 9535205762)</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Data Operations Leadership, SQL Server, ETL, Data Quality, Python Automation, Team Management.</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>Direct email from Richa at Yukthi Techsoft for Head of Data Operations at The Garage India in Bengaluru. Candidate details requested.</t>
+        </is>
+      </c>
+      <c r="O145" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
     <row r="146" ht="33.95" customHeight="1" s="20"/>
     <row r="147" ht="33.95" customHeight="1" s="20"/>
     <row r="148" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Friday Aug 21: Confirmed email and M_Haresh_Kumar_Data_Operations_SQL_PowerBI.pdf sent to Richa for The Garage India Head of Data Operations (Row 145)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Active - High Priority Target (Form Received)</t>
+          <t>Applied - Direct Email &amp; Resume Sent</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Direct email from Richa at Yukthi Techsoft for Head of Data Operations at The Garage India in Bengaluru. Candidate details requested.</t>
+          <t>Direct email response &amp; master resume M_Haresh_Kumar_Data_Operations_SQL_PowerBI.pdf sent to Richa (richa@yukthitech.com) on Fri Aug 21 @ 11:51 AM IST.</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Friday Aug 21: Confirmed official Deloitte SuccessFactors referral email received from RhoHyve AI Labs for Req ID 109094
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9633,7 +9633,7 @@
       </c>
       <c r="H132" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct Recruiter Invite)</t>
+          <t>Referred to Deloitte - Official SuccessFactors Email Received</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -9663,12 +9663,12 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>Applied and confirmed on Naukri for Rhohyve AI Labs Data Governance Consultant (5-10 Yrs) in Bangalore (7.5-17 LPA). 99% match for 15 Yrs Lead, Power BI, DAX, SQL &amp; 0-day notice.</t>
+          <t>Official Deloitte SuccessFactors email received on Fri Aug 21 @ 11:14 AM: Profile referred by RhoHyve AI Labs for Req ID 109094 (Power BI Consultant/Sr Consultant/Manager).</t>
         </is>
       </c>
       <c r="O132" s="29" t="inlineStr">
         <is>
-          <t>Active - Target Applied</t>
+          <t>Active - Official Referral Confirmed</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="H134" s="29" t="inlineStr">
         <is>
-          <t>Active - Eligible to Apply (HYRGPT Platform Active)</t>
+          <t>Referred to Deloitte - Official SuccessFactors Email Received</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9813,12 +9813,12 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>Inspected HYRGPT platform metadata: Requisition is ACTIVE (464 applied of 2,000 limit). Eligible to apply. Core skills: Power BI, DAX, Data Modeling.</t>
+          <t>Official Deloitte SuccessFactors email received on Fri Aug 21 @ 11:14 AM: Profile referred by RhoHyve AI Labs for Req ID 109094 (Power BI Consultant/Sr Consultant/Manager).</t>
         </is>
       </c>
       <c r="O134" s="29" t="inlineStr">
         <is>
-          <t>Active - Target Applied</t>
+          <t>Active - Official Referral Confirmed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Friday Aug 21: Logged Row 146 Orcapod Migration Specialist as Skipped due to Azure DevOps infrastructure skill gap
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O145"/>
+  <dimension ref="A1:O146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10669,7 +10669,83 @@
         </is>
       </c>
     </row>
-    <row r="146" ht="33.95" customHeight="1" s="20"/>
+    <row r="146" ht="33.95" customHeight="1" s="20">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Aug 21, 2026</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Orcapod Consulting Services</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>MS-SQL to Snowflake (Azure) Migration Specialist</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>8-13 Yrs</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>20.0 - 35.0 LPA</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Naukri Email</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Skipped - Infrastructure Migration Skill Gap</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Orcapod Sourcing</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Azure Data Factory (ADF), ADLS Gen2, Azure DevOps, CI/CD, SQL to Snowflake Migration.</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>Skipped per user evaluation: Requiring 8+ Yrs Azure DevOps CI/CD and dedicated cloud infrastructure migration. Out of scope.</t>
+        </is>
+      </c>
+      <c r="O146" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Skipped Infrastructure Role</t>
+        </is>
+      </c>
+    </row>
     <row r="147" ht="33.95" customHeight="1" s="20"/>
     <row r="148" ht="33.95" customHeight="1" s="20"/>
     <row r="149" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Friday Aug 21: Updated Persistent Systems L2 reschedule status to next week per Growel HR update
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -1881,7 +1881,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Reschedule Requested (Pooja / Growel HR Coordinating)</t>
+          <t>Active - L2 Reschedule Pending Next Week</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1911,12 +1911,12 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>Technical glitch reported to Growel HR (Pooja) on WhatsApp @ 12:03 PM. Reschedule email text shared with Pooja @ 12:15 PM; Pooja acknowledged "Ok" @ 12:19 PM to coordinate with Persistent.</t>
-        </is>
-      </c>
-      <c r="O20" s="33" t="inlineStr">
-        <is>
-          <t>Active - Reschedule Requested</t>
+          <t>Pooja (Growel HR) confirmed on Fri Aug 21 @ 12:04 PM: Persistent HR will update L2 reschedule next week. Portal status remains SELECTION.</t>
+        </is>
+      </c>
+      <c r="O20" s="32" t="inlineStr">
+        <is>
+          <t>Active - High Priority</t>
         </is>
       </c>
     </row>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="H129" s="29" t="inlineStr">
         <is>
-          <t>Reschedule Requested (Technical Glitch Email Sent)</t>
+          <t>Active - L2 Reschedule Pending Next Week</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -9438,12 +9438,12 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>Technical glitch occurred (laptop sleep mode) during Q1 at 11:30 AM. Reschedule email sent to careers5@persistent.com &amp; careers2@persistent.com on Wed Aug 19 @ 12:12 PM IST.</t>
-        </is>
-      </c>
-      <c r="O129" s="34" t="inlineStr">
-        <is>
-          <t>Active - Reschedule Requested</t>
+          <t>Pooja (Growel HR) confirmed on Fri Aug 21 @ 12:04 PM: Persistent HR will update L2 reschedule next week. Portal status remains SELECTION.</t>
+        </is>
+      </c>
+      <c r="O129" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Friday Aug 21: Logged Row 147 Indium Software Backend Lead as Skipped (Irrelevant Java/Golang Domain)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O146"/>
+  <dimension ref="A1:O147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10746,7 +10746,83 @@
         </is>
       </c>
     </row>
-    <row r="147" ht="33.95" customHeight="1" s="20"/>
+    <row r="147" ht="33.95" customHeight="1" s="20">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Aug 21, 2026</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Indium Software</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Team Lead (Backend Software Automation - Java/Golang)</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>7-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Naukri Email</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Skipped - Irrelevant Domain (Java/Golang Backend Development)</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Indium Sourcing</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Python, Java, Golang, Shell Scripting, API Integration, Endpoint Security.</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>Irrelevant backend software engineering role requiring Java/Golang/Shell. Matched generic Python &amp; Lead keywords. Skipped.</t>
+        </is>
+      </c>
+      <c r="O147" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Irrelevant Domain</t>
+        </is>
+      </c>
+    </row>
     <row r="148" ht="33.95" customHeight="1" s="20"/>
     <row r="149" ht="33.95" customHeight="1" s="20"/>
     <row r="150" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Friday Aug 21: Confirmed Rhohyve AI Labs VIEWED NAUKRI PROFILE 3 mins ago following Deloitte referral
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -9633,7 +9633,7 @@
       </c>
       <c r="H132" s="29" t="inlineStr">
         <is>
-          <t>Referred to Deloitte - Official SuccessFactors Email Received</t>
+          <t>Active - Deloitte Referral &amp; Naukri Profile Viewed</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -9663,12 +9663,12 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>Official Deloitte SuccessFactors email received on Fri Aug 21 @ 11:14 AM: Profile referred by RhoHyve AI Labs for Req ID 109094 (Power BI Consultant/Sr Consultant/Manager).</t>
+          <t>Rhohyve AI Labs recruiter VIEWED NAUKRI PROFILE on Fri Aug 21 @ 12:52 PM IST following Deloitte SuccessFactors referral submission (Req ID 109094).</t>
         </is>
       </c>
       <c r="O132" s="29" t="inlineStr">
         <is>
-          <t>Active - Official Referral Confirmed</t>
+          <t>Active - High Priority</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Friday Aug 21: Logged Row 148 EY Data Modeller Manager as Skipped per BGV degree evaluation
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O147"/>
+  <dimension ref="A1:O148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10823,7 +10823,83 @@
         </is>
       </c>
     </row>
-    <row r="148" ht="33.95" customHeight="1" s="20"/>
+    <row r="148" ht="33.95" customHeight="1" s="20">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Aug 21, 2026</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>EY (Ernst &amp; Young)</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Data Modeller - Manager</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>9-14 Yrs</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Naukri Feed</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Skipped - Big-4 HR BGV Graduation Degree Policy</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>0 Days</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>EY Sourcing</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Data Modeling, Data Modeling Architecture, ETL, ERwin, ER Studio.</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Skipped per user evaluation regarding Big-4 HR BGV degree verification policies.</t>
+        </is>
+      </c>
+      <c r="O148" s="31" t="inlineStr">
+        <is>
+          <t>Inactive - Skipped BGV Policy</t>
+        </is>
+      </c>
+    </row>
     <row r="149" ht="33.95" customHeight="1" s="20"/>
     <row r="150" ht="33.95" customHeight="1" s="20"/>
     <row r="151" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Friday Aug 21: Logged Row 149 BCT Consulting Data Engineer F2F Bangalore
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O148"/>
+  <dimension ref="A1:O149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10900,7 +10900,83 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="33.95" customHeight="1" s="20"/>
+    <row r="149" ht="33.95" customHeight="1" s="20">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Aug 21, 2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BCT Consulting</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Data Engineer (F2F Interview - Bangalore)</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>7-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>5.0 - 12.0 LPA</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Naukri Applied</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Applied - Direct Mailer Applied</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>BCT Consulting Sourcing</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ETL, Python, SQL, Data Warehousing, Data Cleansing, Data Validation.</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>Applied on Naukri for Data Engineer F2F Interview Drive in Bangalore via BCT Consulting.</t>
+        </is>
+      </c>
+      <c r="O149" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="150" ht="33.95" customHeight="1" s="20"/>
     <row r="151" ht="33.95" customHeight="1" s="20"/>
     <row r="152" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Friday Aug 21: Confirmed recruiter NVite received from Pooja (BCT Consulting) for Data Engineer F2F (Row 149)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10938,7 +10938,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Applied - Direct Mailer Applied</t>
+          <t>Applied - Recruiter NVite Received from Pooja</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Applied on Naukri for Data Engineer F2F Interview Drive in Bangalore via BCT Consulting.</t>
+          <t>Pooja (BCT Consulting) SENT RECRUITER NVITE on Naukri on Fri Aug 21 @ 02:32 PM IST for Data Engineer F2F Bangalore.</t>
         </is>
       </c>
       <c r="O149" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Saturday Aug 22: Audited and filtered job sheet statuses. Deprioritized walk-in/degree-filtered roles and highlighted active targets.
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -8763,12 +8763,12 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>Direct recruiter NVite received from Chanya Roheda (Xponentium) on Thu Aug 13 @ 10:52 AM. Applied and confirmed for Snowflake Developer in Bengaluru/Hyderabad/Pune.</t>
-        </is>
-      </c>
-      <c r="O120" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Applied</t>
+          <t>Walk-in gate Codility pre-test filter mismatch on Aug 22. Review if HR contacts directly.</t>
+        </is>
+      </c>
+      <c r="O120" s="34" t="inlineStr">
+        <is>
+          <t>Deprioritized - Review If Called</t>
         </is>
       </c>
     </row>
@@ -10121,12 +10121,12 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>Skipped per user explicit preference: User not interested in outside India / international staffing agency postings.</t>
-        </is>
-      </c>
-      <c r="O138" s="31" t="inlineStr">
-        <is>
-          <t>Inactive - Skipped Staffing Agency</t>
+          <t>Walk-in gate Codility pre-test filter mismatch on Aug 22. Review if HR contacts directly.</t>
+        </is>
+      </c>
+      <c r="O138" s="34" t="inlineStr">
+        <is>
+          <t>Deprioritized - Review If Called</t>
         </is>
       </c>
     </row>
@@ -10275,12 +10275,12 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>Krati Sarin (Co-Founder @ Orcapod) DOWNLOADED RESUME 43 minutes ago on Naukri following prescreening email submission.</t>
+          <t>Prescreening form submitted. Krati Sarin downloaded CV on Naukri.</t>
         </is>
       </c>
       <c r="O140" s="29" t="inlineStr">
         <is>
-          <t>Active - High Priority</t>
+          <t>Active - High Priority Target</t>
         </is>
       </c>
     </row>
@@ -10352,7 +10352,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>Application &amp; screening questions confirmed submitted on Naukri on Thu Aug 20 @ 3:20 PM IST (Immediate Joiner / 15 Yrs IT Exp).</t>
+          <t>Screening submitted on Naukri.</t>
         </is>
       </c>
       <c r="O141" s="29" t="inlineStr">
@@ -10429,12 +10429,12 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>Irrelevant electrical engineering job mailer. Matched word Power System instead of Power BI. Skipped.</t>
+          <t>Electrical power system engineering role out of scope.</t>
         </is>
       </c>
       <c r="O142" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Irrelevant Domain</t>
+          <t>Skipped - Irrelevant Role</t>
         </is>
       </c>
     </row>
@@ -10506,12 +10506,12 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>Recruiter email received from Monisha Devi (O2F Info Solutions). Skipped as deployment is on O2F payroll (contract) and user prefers permanent FTE roles.</t>
+          <t>Vendor C2H contract deployment for Infosys. User prefers direct FTE.</t>
         </is>
       </c>
       <c r="O143" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Skipped Contract</t>
+          <t>Skipped - Vendor Contract</t>
         </is>
       </c>
     </row>
@@ -10583,12 +10583,12 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>WhatsApp conversation completed @ 17:21. Candidate politely declined QA testing JD. Rahul acknowledged "ok".</t>
+          <t>QA software testing role out of scope. Politely declined on WhatsApp.</t>
         </is>
       </c>
       <c r="O144" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Closed</t>
+          <t>Closed - QA Testing Out of Scope</t>
         </is>
       </c>
     </row>
@@ -10660,7 +10660,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Direct email response &amp; master resume M_Haresh_Kumar_Data_Operations_SQL_PowerBI.pdf sent to Richa (richa@yukthitech.com) on Fri Aug 21 @ 11:51 AM IST.</t>
+          <t>Head of Data Ops role. Application &amp; resume sent to Richa (richa@yukthitech.com).</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">
@@ -10737,12 +10737,12 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>Skipped per user evaluation: Requiring 8+ Yrs Azure DevOps CI/CD and dedicated cloud infrastructure migration. Out of scope.</t>
+          <t>Azure DevOps CI/CD infrastructure skill gap.</t>
         </is>
       </c>
       <c r="O146" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Skipped Infrastructure Role</t>
+          <t>Skipped - CI/CD Infrastructure Gap</t>
         </is>
       </c>
     </row>
@@ -10814,12 +10814,12 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>Irrelevant backend software engineering role requiring Java/Golang/Shell. Matched generic Python &amp; Lead keywords. Skipped.</t>
+          <t>Java/Golang backend role. Clicked Not Interested on Naukri.</t>
         </is>
       </c>
       <c r="O147" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Irrelevant Domain</t>
+          <t>Skipped - Irrelevant Backend Role</t>
         </is>
       </c>
     </row>
@@ -10891,12 +10891,12 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>Skipped per user evaluation regarding Big-4 HR BGV degree verification policies.</t>
+          <t>Big-4 HR background verification degree policy filter.</t>
         </is>
       </c>
       <c r="O148" s="31" t="inlineStr">
         <is>
-          <t>Inactive - Skipped BGV Policy</t>
+          <t>Skipped - Degree Policy Filter</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Pooja (BCT Consulting) SENT RECRUITER NVITE on Naukri on Fri Aug 21 @ 02:32 PM IST for Data Engineer F2F Bangalore.</t>
+          <t>Recruiter NVite received from Pooja (BCT Consulting) for Data Engineer F2F.</t>
         </is>
       </c>
       <c r="O149" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Saturday Aug 22: Logged Row 150 Deloitte SAP BODS Consultant as Skipped (Out of scope SAP tool)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O149"/>
+  <dimension ref="A1:O150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10977,7 +10977,83 @@
         </is>
       </c>
     </row>
-    <row r="150" ht="33.95" customHeight="1" s="20"/>
+    <row r="150" ht="33.95" customHeight="1" s="20">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Deloitte US-India Offices</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>SAP BODS Consultant</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>12-16 Yrs</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad / Chennai</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Naukri Mailer (Skipped)</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Skipped - Out of Scope</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Deloitte Sourcing</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>SAP BODS, SAP BW, Data Migration, ETL Implementation.</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Proprietary SAP BODS/BW ETL tool role out of scope. User clicked Not Interested.</t>
+        </is>
+      </c>
+      <c r="O150" s="31" t="inlineStr">
+        <is>
+          <t>Skipped - SAP Tool Out of Scope</t>
+        </is>
+      </c>
+    </row>
     <row r="151" ht="33.95" customHeight="1" s="20"/>
     <row r="152" ht="33.95" customHeight="1" s="20"/>
     <row r="153" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Saturday Aug 22: Logged Rows 151 (Kcyber Experts Contact Viewed) & 152 (Ingenium Digital NVite Received)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O150"/>
+  <dimension ref="A1:O152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -11054,8 +11054,160 @@
         </is>
       </c>
     </row>
-    <row r="151" ht="33.95" customHeight="1" s="20"/>
-    <row r="152" ht="33.95" customHeight="1" s="20"/>
+    <row r="151" ht="33.95" customHeight="1" s="20">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Kcyber Experts</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Data Operations / Analytics Lead</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>10-15 Yrs</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Nagpur / Remote</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Search</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Recruiter Viewed Contact</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Kcyber Experts HR</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Data Operations, SQL, Power BI, Analytics.</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Kcyber Experts HR recruiter VIEWED CONTACT DETAILS on Naukri on Sat Aug 22 @ 10:30 AM IST.</t>
+        </is>
+      </c>
+      <c r="O151" s="29" t="inlineStr">
+        <is>
+          <t>Active - Recruiter Sourced</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="33.95" customHeight="1" s="20">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Ingenium Digital</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Analytics / Power BI Lead</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>10-15 Yrs</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Naukri NVite</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Recruiter NVite Received</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Samhitha Gowda (Ingenium Digital)</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Power BI, SQL, DAX, Data Analytics.</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>Samhitha Gowda (Ingenium Digital) SENT RECRUITER NVITE on Naukri for Analytics Lead role.</t>
+        </is>
+      </c>
+      <c r="O152" s="29" t="inlineStr">
+        <is>
+          <t>Active - Recruiter Sourced</t>
+        </is>
+      </c>
+    </row>
     <row r="153" ht="33.95" customHeight="1" s="20"/>
     <row r="154" ht="33.95" customHeight="1" s="20"/>
     <row r="155" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Saturday Aug 22: Logged 4 top matching targets: WinWire Tech Lead (Row 153), Recruito Remote BI Lead (Row 154), VML ES Data Lead (Row 155), Virtusa Senior DE (Row 156)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O152"/>
+  <dimension ref="A1:O156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -11208,10 +11208,314 @@
         </is>
       </c>
     </row>
-    <row r="153" ht="33.95" customHeight="1" s="20"/>
-    <row r="154" ht="33.95" customHeight="1" s="20"/>
-    <row r="155" ht="33.95" customHeight="1" s="20"/>
-    <row r="156" ht="33.95" customHeight="1" s="20"/>
+    <row r="153" ht="33.95" customHeight="1" s="20">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>WinWire</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Technical Lead / Sr Technical Lead - Power BI, SQL</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>9-14 Yrs</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Naukri Search Sourced</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Target Identified</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>WinWire Sourcing</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Power BI, SQL, DAX, Data Modeling, Data Warehouse concepts.</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>100% Target Match! Power BI, SQL, DAX, Data Modeling Tech Lead in Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O153" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="33.95" customHeight="1" s="20">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Recruito</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Power BI Lead (Remote)</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>8-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>30.0 - 37.5 LPA</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Naukri Search Sourced</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Target Identified</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Recruito HR</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Power BI, Data Modeling, Leading BI Development teams.</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>100% Target Match! Remote Power BI Lead role (30-37.5 LPA).</t>
+        </is>
+      </c>
+      <c r="O154" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="33.95" customHeight="1" s="20">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>VML ES</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Data Lead</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>10-15 Yrs</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Naukri Search Sourced</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Target Identified</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>VML ES Sourcing</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Business Intelligence, Power BI, Data Strategy, Data Governance, SQL.</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>100% Target Match! Business Intelligence &amp; Data Governance Lead in Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O155" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="33.95" customHeight="1" s="20">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Aug 22, 2026</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Virtusa</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>9-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>1.0 - 30.0 LPA</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Naukri Search Sourced</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Target Identified</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Virtusa Sourcing</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Snowflake, Data Engineering, Data Build Tool, Data Warehousing.</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>100% Target Match! Snowflake Data Engineering role at Virtusa Bengaluru.</t>
+        </is>
+      </c>
+      <c r="O156" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
     <row r="157" ht="33.95" customHeight="1" s="20"/>
     <row r="158" ht="33.95" customHeight="1" s="20"/>
     <row r="159" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Saturday Aug 22: Application & screening questionnaire submitted on Naukri for Virtusa Senior Data Engineer (Row 156)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11477,7 +11477,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Target Identified</t>
+          <t>Applied - Screening Completed</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -11507,12 +11507,12 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>100% Target Match! Snowflake Data Engineering role at Virtusa Bengaluru.</t>
+          <t>Application submitted on Naukri on Sat Aug 22 @ 01:54 PM IST. Screening questionnaire completed (Relocate: Yes, Snowflake: &lt;9 yrs, Senior DE: &lt;9 yrs).</t>
         </is>
       </c>
       <c r="O156" s="29" t="inlineStr">
         <is>
-          <t>Active - High Priority Target</t>
+          <t>Active - Target Applied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Saturday Aug 22: Updated real-time Naukri recruiter activity. HCLTech & Yukthi recruiters active TODAY.
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Applied - Direct Email &amp; Resume Sent</t>
+          <t>Resume Viewed - Recruiter Active TODAY</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10660,12 +10660,12 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Head of Data Ops role. Application &amp; resume sent to Richa (richa@yukthitech.com).</t>
+          <t>Yukthi Systems (Head of Data Ops) recruiter viewed resume. Recruiter active TODAY (Sat Aug 22).</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">
         <is>
-          <t>Active - High Priority Target</t>
+          <t>Active - Recruiter Sourced</t>
         </is>
       </c>
     </row>
@@ -11477,7 +11477,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Applied - Screening Completed</t>
+          <t>Application Sent Today</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -11507,12 +11507,12 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>Application submitted on Naukri on Sat Aug 22 @ 01:54 PM IST. Screening questionnaire completed (Relocate: Yes, Snowflake: &lt;9 yrs, Senior DE: &lt;9 yrs).</t>
+          <t>Virtusa Senior Data Engineer application sent today (Sat Aug 22). Recruiter active 1d ago.</t>
         </is>
       </c>
       <c r="O156" s="29" t="inlineStr">
         <is>
-          <t>Active - Target Applied</t>
+          <t>Active - Recruiter Sourced</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Saturday Aug 22: Logged 100% target match McAfee Data Engineer / Analyst (Req 1469) as Row 157
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O156"/>
+  <dimension ref="A1:O157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -11516,7 +11516,78 @@
         </is>
       </c>
     </row>
-    <row r="157" ht="33.95" customHeight="1" s="20"/>
+    <row r="157" ht="33.95" customHeight="1" s="20">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>McAfee</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Data Engineer / Analyst (Req 1469)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>LinkedIn Search</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Bengaluru Hybrid</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Direct LinkedIn</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Target Selected</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>6-8 Yrs</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>SQL, Power BI, Data Quality, Operational Analytics</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Direct Link</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>LinkedIn Sourced</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>100% Target Match for SQL, Power BI, Data Quality &amp; Operational Analytics. LinkedIn Match Status: GOOD.</t>
+        </is>
+      </c>
+      <c r="O157" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Logged</t>
+        </is>
+      </c>
+    </row>
     <row r="158" ht="33.95" customHeight="1" s="20"/>
     <row r="159" ht="33.95" customHeight="1" s="20"/>
     <row r="160" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Saturday Aug 22: Filling McAfee candidate profile form on Workday portal (Row 157)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11554,7 +11554,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Target Selected</t>
+          <t>Application Form In Progress</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -11579,12 +11579,12 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>100% Target Match for SQL, Power BI, Data Quality &amp; Operational Analytics. LinkedIn Match Status: GOOD.</t>
+          <t>Filling candidate profile application form on McAfee Workday portal (Req 1469) on Sat Aug 22 @ 04:21 PM IST.</t>
         </is>
       </c>
       <c r="O157" s="29" t="inlineStr">
         <is>
-          <t>Active - Target Logged</t>
+          <t>Active - Form In Progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Saturday Aug 22: Application submitted successfully on official Workday portal for McAfee Data Engineer / Analyst (Row 157)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11554,7 +11554,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Application Form In Progress</t>
+          <t>Applied - Official Portal Submitted</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -11579,12 +11579,12 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>Filling candidate profile application form on McAfee Workday portal (Req 1469) on Sat Aug 22 @ 04:21 PM IST.</t>
+          <t>Application submitted successfully on McAfee Workday Portal (Req 2026-1469) on Sat Aug 22 @ 04:23 PM IST. Target Match: 100% (SQL, Power BI, Data Quality).</t>
         </is>
       </c>
       <c r="O157" s="29" t="inlineStr">
         <is>
-          <t>Active - Form In Progress</t>
+          <t>Active - Target Applied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Logged fresh Naukri NVite from Blas-connect IT Services as Row 158 and updated Yukthi email correction
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O157"/>
+  <dimension ref="A1:O158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -10660,7 +10660,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Yukthi Systems (Head of Data Ops) recruiter viewed resume. Recruiter active TODAY (Sat Aug 22).</t>
+          <t>Delivery retry warning received for .org domain. Correct email is richa@yukthitech.com. WhatsApp follow-up queued for 9535205762.</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">
@@ -11588,7 +11588,83 @@
         </is>
       </c>
     </row>
-    <row r="158" ht="33.95" customHeight="1" s="20"/>
+    <row r="158" ht="33.95" customHeight="1" s="20">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Blas-connect IT Services</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Data Operations / Senior DE Lead</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>10-15 Yrs</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>16.0 - 18.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Naukri NVite</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>NVite Received - Action Required</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>HR Recruiter (Blas-connect)</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Data Operations, SQL, Power BI, Cloud Pipelines, Team Management</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>Naukri NVite received 9h ago on Monday Aug 24 morning. Direct recruiter outreach.</t>
+        </is>
+      </c>
+      <c r="O158" s="29" t="inlineStr">
+        <is>
+          <t>Active - NVite Received</t>
+        </is>
+      </c>
+    </row>
     <row r="159" ht="33.95" customHeight="1" s="20"/>
     <row r="160" ht="33.95" customHeight="1" s="20"/>
     <row r="161" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Monday Aug 24: Updated Row 158 to Skipped - Location Mismatch (Hyderabad) for Blas-connect Finance Analytics Manager
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11596,12 +11596,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Blas-connect IT Services</t>
+          <t>Blas-connect IT Services (Foreign MNC)</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Data Operations / Senior DE Lead</t>
+          <t>Senior Manager, Finance Analytics &amp; Insights</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -11611,7 +11611,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Hyderabad (Hybrid)</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>NVite Received - Action Required</t>
+          <t>Skipped - Location Mismatch (Hyderabad)</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -11656,12 +11656,12 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>Naukri NVite received 9h ago on Monday Aug 24 morning. Direct recruiter outreach.</t>
-        </is>
-      </c>
-      <c r="O158" s="29" t="inlineStr">
-        <is>
-          <t>Active - NVite Received</t>
+          <t>Role requires physical hybrid presence in Hyderabad and specialized Controllership/SOX domain focus. Location mismatch vs Bengaluru target.</t>
+        </is>
+      </c>
+      <c r="O158" s="34" t="inlineStr">
+        <is>
+          <t>Skipped - Location Mismatch</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Confirmed SELECTION status on Persistent Systems portal for Senior Data Engineer (Row 68)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -5069,7 +5069,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Profile Viewed</t>
+          <t>Selection - L2 Reschedule Pending</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -5099,12 +5099,12 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>Naukri profile view logged from ATS Mohali Head HR.</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>Active - Profile Viewed</t>
+          <t>Candidate portal status officially marked SELECTION for Senior Data Engineer! Activity feed confirms Interview Confirmed - L2. Growel HR (Pooja) rescheduling slot for week of Aug 24-28.</t>
+        </is>
+      </c>
+      <c r="O68" s="29" t="inlineStr">
+        <is>
+          <t>Active - Selection / L2 Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Richa (Yukthi Techsoft) responded on WhatsApp requesting candidate details for Head of Data Operations (Row 145)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Resume Viewed - Recruiter Active TODAY</t>
+          <t>Recruiter Responded - Details Requested</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Delivery retry warning received for .org domain. Correct email is richa@yukthitech.com. WhatsApp follow-up queued for 9535205762.</t>
+          <t>Richa (+91-9535205762) responded on WhatsApp on Mon Aug 24 @ 11:36 AM IST requesting candidate details &amp; updated CV for Head of Data Operations role.</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Monday Aug 24: Candidate details & resume submitted on WhatsApp to Richa for Head of Data Operations (Row 145)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Recruiter Responded - Details Requested</t>
+          <t>Details Submitted via WhatsApp</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Richa (+91-9535205762) responded on WhatsApp on Mon Aug 24 @ 11:36 AM IST requesting candidate details &amp; updated CV for Head of Data Operations role.</t>
+          <t>Candidate details &amp; resume submitted on WhatsApp to Richa (+91-9535205762) for Head of Data Operations on Mon Aug 24 @ 11:39 AM IST.</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Monday Aug 24: Richa confirmed profile under processing for The Garage Head of Data Operations (Row 145)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Details Submitted via WhatsApp</t>
+          <t>Profile Under Process - Recruiter Confirmed</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10660,12 +10660,12 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Candidate details &amp; resume submitted on WhatsApp to Richa (+91-9535205762) for Head of Data Operations on Mon Aug 24 @ 11:39 AM IST.</t>
+          <t>Richa (+91-9535205762) confirmed on WhatsApp (Mon Aug 24 @ 11:46 AM IST): Thankyou for sharing the details and resume. We will process again and update you asap.</t>
         </is>
       </c>
       <c r="O145" s="29" t="inlineStr">
         <is>
-          <t>Active - Recruiter Sourced</t>
+          <t>Active - Profile Under Process</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Deprioritized Deloitte SAP BODS role (Row 150) due to niche SAP BODS/BAPI requirement
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11015,7 +11015,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Skipped - Out of Scope</t>
+          <t>Skipped - SAP BODS/BAPI Specialty</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -11045,12 +11045,12 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>Proprietary SAP BODS/BW ETL tool role out of scope. User clicked Not Interested.</t>
-        </is>
-      </c>
-      <c r="O150" s="31" t="inlineStr">
-        <is>
-          <t>Skipped - SAP Tool Out of Scope</t>
+          <t>Role requires specialized SAP BODS / BAPI programming language expertise. Deprioritized vs core Data Ops &amp; Snowflake/SQL targets.</t>
+        </is>
+      </c>
+      <c r="O150" s="34" t="inlineStr">
+        <is>
+          <t>Deprioritized - Niche Skill</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Audited 40+ Naukri roles; logged Rows 159 (Recruito Remote Power BI Lead), 160 (Prorsum Snowflake DE Bengaluru), 161 (Blackbuck Remote Sr DE)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O158"/>
+  <dimension ref="A1:O161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -11665,9 +11665,237 @@
         </is>
       </c>
     </row>
-    <row r="159" ht="33.95" customHeight="1" s="20"/>
-    <row r="160" ht="33.95" customHeight="1" s="20"/>
-    <row r="161" ht="33.95" customHeight="1" s="20"/>
+    <row r="159" ht="33.95" customHeight="1" s="20">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Recruito</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Power BI Lead</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>8-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>30.0 - 37.5 LPA</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Naukri Sourced</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Active Target - Remote Lead</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Recruito Talent Team</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Power BI, DAX, Data Modeling, Azure Data Factory, Power Apps, Executive Dashboards</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>100% Target Match for Power BI Lead &amp; Data Modeling (Remote 30-37.5 LPA).</t>
+        </is>
+      </c>
+      <c r="O159" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Sourced</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="33.95" customHeight="1" s="20">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Prorsum Technologies</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Snowflake Data Engineer</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>8-13 Yrs</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Bengaluru Hybrid</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>16.0 - 22.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Naukri Sourced</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Active Target - Snowflake DE</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Prorsum Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Snowflake, Advanced SQL, Data Engineering, ETL, Data Warehousing, Data Modeling</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>100% Target Match for Snowflake &amp; Advanced SQL (Bengaluru Hybrid). Posted 2 days ago.</t>
+        </is>
+      </c>
+      <c r="O160" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Sourced</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="33.95" customHeight="1" s="20">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Blackbuck Insights (BBI)</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Sr Data Engineer (dbt / SQL / Snowflake)</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>10-15 Yrs</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>20.0 - 28.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Naukri Sourced</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Active Target - Remote Sr DE</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Blackbuck Recruitment Team</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Data Engineering, Data Quality, Version Control, SQL, Stored Procedures, Data Warehousing</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>100% Target Match for Senior Data Engineer &amp; Data Quality (Remote). Posted 6 days ago.</t>
+        </is>
+      </c>
+      <c r="O161" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Sourced</t>
+        </is>
+      </c>
+    </row>
     <row r="162" ht="33.95" customHeight="1" s="20"/>
     <row r="163" ht="33.95" customHeight="1" s="20"/>
     <row r="164" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Monday Aug 24: Confirmed 100% match for Prorsum Snowflake Data Engineer (Row 160) matching 4 Snowflake Badges
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11780,7 +11780,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Active Target - Snowflake DE</t>
+          <t>Active Target - Snowflake Certified Match</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -11810,7 +11810,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>100% Target Match for Snowflake &amp; Advanced SQL (Bengaluru Hybrid). Posted 2 days ago.</t>
+          <t>100% Target Match for Prorsum Technologies Snowflake Data Engineer (8-13 Yrs, Bengaluru). Matches 4 Earned Snowflake Badges on resume!</t>
         </is>
       </c>
       <c r="O160" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Monday Aug 24: Updated Row 160 Prorsum note to reflect 4 Snowflake Badges vs SnowPro readiness
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11780,7 +11780,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Active Target - Snowflake Certified Match</t>
+          <t>Active Target - Snowflake Badges (SnowPro Preferred)</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -11810,12 +11810,12 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>100% Target Match for Prorsum Technologies Snowflake Data Engineer (8-13 Yrs, Bengaluru). Matches 4 Earned Snowflake Badges on resume!</t>
-        </is>
-      </c>
-      <c r="O160" s="29" t="inlineStr">
-        <is>
-          <t>Active - Target Sourced</t>
+          <t>JD mandates Snowflake Certification. Candidate holds 4 Snowflake Hands-On Essentials Badges. Prepared to state badges + SnowPro readiness.</t>
+        </is>
+      </c>
+      <c r="O160" s="34" t="inlineStr">
+        <is>
+          <t>Active - Credentials Match</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Updated Row 160 Prorsum to Skipped - Mandatory SnowPro Cert Required
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -11780,7 +11780,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Active Target - Snowflake Badges (SnowPro Preferred)</t>
+          <t>Skipped - SnowPro Core Mandatory</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -11810,12 +11810,12 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>JD mandates Snowflake Certification. Candidate holds 4 Snowflake Hands-On Essentials Badges. Prepared to state badges + SnowPro readiness.</t>
+          <t>Portal strictly requires formal proctored SnowPro Core certification. Candidate answered No (holds 4 Hands-On Badges). Role skipped to avoid portal mismatch.</t>
         </is>
       </c>
       <c r="O160" s="34" t="inlineStr">
         <is>
-          <t>Active - Credentials Match</t>
+          <t>Skipped - Mandatory Cert</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday Aug 24: Logged fresh 100% target match Virtusa Senior Data Engineer (3 Openings, Graduation Not Required) as Row 162
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O161"/>
+  <dimension ref="A1:O162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -11896,7 +11896,83 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="33.95" customHeight="1" s="20"/>
+    <row r="162" ht="33.95" customHeight="1" s="20">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Virtusa</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer (Financial Services - 3 Openings)</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>9-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>16.0 - 24.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Naukri Sourced</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Active Target - Fresh 3 Openings</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Virtusa Talent Team</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Snowflake (stages, views, roles), SQL (window funcs, joins), Python ETL, Data Quality, Financial Services</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>100% Target Match for Virtusa Senior DE (3 Openings, Posted JUST NOW). Graduation Not Required. Financial Services domain.</t>
+        </is>
+      </c>
+      <c r="O162" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Sourced</t>
+        </is>
+      </c>
+    </row>
     <row r="163" ht="33.95" customHeight="1" s="20"/>
     <row r="164" ht="33.95" customHeight="1" s="20"/>
     <row r="165" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Monday Aug 24: Applied to Virtusa Senior DE (Row 162) and skipped Walmart BPO role (Row 163)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O162"/>
+  <dimension ref="A1:O163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -11934,7 +11934,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Active Target - Fresh 3 Openings</t>
+          <t>Applied - Screening Completed</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -11964,16 +11964,92 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>100% Target Match for Virtusa Senior DE (3 Openings, Posted JUST NOW). Graduation Not Required. Financial Services domain.</t>
+          <t>Application and screening questionnaire completed on Naukri on Mon Aug 24 @ 12:18 PM IST (3 Openings, Financial Services).</t>
         </is>
       </c>
       <c r="O162" s="29" t="inlineStr">
         <is>
-          <t>Active - Target Sourced</t>
-        </is>
-      </c>
-    </row>
-    <row r="163" ht="33.95" customHeight="1" s="20"/>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="33.95" customHeight="1" s="20">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Team Lead (BPO / Customer Success)</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>6-12 Yrs</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>8.0 - 13.0 LPA</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Naukri Sourced</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Skipped - BPO / Customer Service Domain</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Walmart Recruitment Team</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>BPO Operations, Attrition Control, Shrinkage, Call Center Customer Success</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>Call center / BPO operations role. Mismatch vs Data Operations &amp; Analytics Leadership target.</t>
+        </is>
+      </c>
+      <c r="O163" s="34" t="inlineStr">
+        <is>
+          <t>Skipped - BPO Domain</t>
+        </is>
+      </c>
+    </row>
     <row r="164" ht="33.95" customHeight="1" s="20"/>
     <row r="165" ht="33.95" customHeight="1" s="20"/>
     <row r="166" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Monday Aug 24: Logged 100% target match EXL Service Remote Data Engineer (Posted 24 MINS AGO on LinkedIn) as Row 164
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O163"/>
+  <dimension ref="A1:O164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -12050,7 +12050,83 @@
         </is>
       </c>
     </row>
-    <row r="164" ht="33.95" customHeight="1" s="20"/>
+    <row r="164" ht="33.95" customHeight="1" s="20">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>EXL Service</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Data Engineer / Analytics Engineer</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>5+ Yrs</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Remote (India)</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>22.0 - 32.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Active High Priority - Posted 24m Ago</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>0 Days (Immediate)</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>EXL Talent Acquisition / Rishabh Pandey</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Snowflake, dbt Cloud, Fivetran, Advanced SQL, Claude Code AI Workflows, Data Modeling, Data Quality</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>100% Target Match! Posted 24 MINS AGO on LinkedIn. Easy Apply available. Explicitly mandates Claude Code &amp; AI coding workflows!</t>
+        </is>
+      </c>
+      <c r="O164" s="29" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
     <row r="165" ht="33.95" customHeight="1" s="20"/>
     <row r="166" ht="33.95" customHeight="1" s="20"/>
     <row r="167" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Monday Aug 24: Application submitted via LinkedIn Easy Apply for EXL Service Remote Data Engineer (Row 164)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -12088,7 +12088,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Active High Priority - Posted 24m Ago</t>
+          <t>Applied - LinkedIn Easy Apply</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -12118,12 +12118,12 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>100% Target Match! Posted 24 MINS AGO on LinkedIn. Easy Apply available. Explicitly mandates Claude Code &amp; AI coding workflows!</t>
+          <t>Application submitted via LinkedIn Easy Apply within 25 mins of posting for EXL Service Remote Data Engineer on Mon Aug 24 @ 01:18 PM IST.</t>
         </is>
       </c>
       <c r="O164" s="29" t="inlineStr">
         <is>
-          <t>Active - High Priority Target</t>
+          <t>Active - Target Applied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate Revenue Leakage Calculator to permanent GitHub Pages hosting and fix broken GoDaddy parked domain
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -78,6 +78,10 @@
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="18">
@@ -180,7 +184,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -233,12 +237,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -312,6 +330,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -745,7 +769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O164"/>
+  <dimension ref="A1:O182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -12127,24 +12151,1356 @@
         </is>
       </c>
     </row>
-    <row r="165" ht="33.95" customHeight="1" s="20"/>
-    <row r="166" ht="33.95" customHeight="1" s="20"/>
-    <row r="167" ht="33.95" customHeight="1" s="20"/>
-    <row r="168" ht="33.95" customHeight="1" s="20"/>
-    <row r="169" ht="33.95" customHeight="1" s="20"/>
-    <row r="170" ht="33.95" customHeight="1" s="20"/>
-    <row r="171" ht="33.95" customHeight="1" s="20"/>
-    <row r="172" ht="33.95" customHeight="1" s="20"/>
-    <row r="173" ht="33.95" customHeight="1" s="20"/>
-    <row r="174" ht="33.95" customHeight="1" s="20"/>
-    <row r="175" ht="33.95" customHeight="1" s="20"/>
-    <row r="176" ht="33.95" customHeight="1" s="20"/>
-    <row r="177" ht="33.95" customHeight="1" s="20"/>
-    <row r="178" ht="33.95" customHeight="1" s="20"/>
-    <row r="179" ht="33.95" customHeight="1" s="20"/>
-    <row r="180" ht="33.95" customHeight="1" s="20"/>
-    <row r="181" ht="33.95" customHeight="1" s="20"/>
-    <row r="182" ht="33.95" customHeight="1" s="20"/>
+    <row r="165" ht="33.95" customHeight="1" s="20">
+      <c r="A165" s="35" t="inlineStr">
+        <is>
+          <t>Aug 26, 2026</t>
+        </is>
+      </c>
+      <c r="B165" s="36" t="inlineStr">
+        <is>
+          <t>Coforge</t>
+        </is>
+      </c>
+      <c r="C165" s="36" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="D165" s="36" t="inlineStr">
+        <is>
+          <t>Bangalore / Hybrid</t>
+        </is>
+      </c>
+      <c r="E165" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F165" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G165" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Snowflake_Data_Engineer_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H165" s="35" t="inlineStr">
+        <is>
+          <t>Contacted by Email</t>
+        </is>
+      </c>
+      <c r="I165" s="36" t="inlineStr">
+        <is>
+          <t>HR Team</t>
+        </is>
+      </c>
+      <c r="J165" s="36" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="K165" s="36" t="inlineStr">
+        <is>
+          <t>Initial Outreach</t>
+        </is>
+      </c>
+      <c r="L165" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M165" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N165" s="36" t="inlineStr">
+        <is>
+          <t>Recruiter contacted by email for senior data pipeline role.</t>
+        </is>
+      </c>
+      <c r="O165" s="35" t="inlineStr">
+        <is>
+          <t>Active - In Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="33.95" customHeight="1" s="20">
+      <c r="A166" s="35" t="inlineStr">
+        <is>
+          <t>Aug 31, 2026</t>
+        </is>
+      </c>
+      <c r="B166" s="36" t="inlineStr">
+        <is>
+          <t>Seventh Edge Consulting Services</t>
+        </is>
+      </c>
+      <c r="C166" s="36" t="inlineStr">
+        <is>
+          <t>Sr Data Modeler</t>
+        </is>
+      </c>
+      <c r="D166" s="36" t="inlineStr">
+        <is>
+          <t>Pune / Gurgaon / Bangalore</t>
+        </is>
+      </c>
+      <c r="E166" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F166" s="35" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G166" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H166" s="35" t="inlineStr">
+        <is>
+          <t>Application Viewed</t>
+        </is>
+      </c>
+      <c r="I166" s="36" t="inlineStr">
+        <is>
+          <t>Recruiter Team</t>
+        </is>
+      </c>
+      <c r="J166" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K166" s="36" t="inlineStr">
+        <is>
+          <t>Application Review</t>
+        </is>
+      </c>
+      <c r="L166" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M166" s="36" t="inlineStr">
+        <is>
+          <t>14-16 LPA</t>
+        </is>
+      </c>
+      <c r="N166" s="36" t="inlineStr">
+        <is>
+          <t>Application viewed by recruiter 7 days ago, recruiter active.</t>
+        </is>
+      </c>
+      <c r="O166" s="35" t="inlineStr">
+        <is>
+          <t>Active - Viewed</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="33.95" customHeight="1" s="20">
+      <c r="A167" s="35" t="inlineStr">
+        <is>
+          <t>Sep 01, 2026</t>
+        </is>
+      </c>
+      <c r="B167" s="36" t="inlineStr">
+        <is>
+          <t>Anblicks Solutions</t>
+        </is>
+      </c>
+      <c r="C167" s="36" t="inlineStr">
+        <is>
+          <t>Senior Platform Engineer (Snowflake &amp; Oracle)</t>
+        </is>
+      </c>
+      <c r="D167" s="36" t="inlineStr">
+        <is>
+          <t>Ahmedabad / Bangalore</t>
+        </is>
+      </c>
+      <c r="E167" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F167" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G167" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Snowflake_Data_Engineer_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H167" s="35" t="inlineStr">
+        <is>
+          <t>Application Viewed</t>
+        </is>
+      </c>
+      <c r="I167" s="36" t="inlineStr">
+        <is>
+          <t>Veeraiah J</t>
+        </is>
+      </c>
+      <c r="J167" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K167" s="36" t="inlineStr">
+        <is>
+          <t>Application Review</t>
+        </is>
+      </c>
+      <c r="L167" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M167" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N167" s="36" t="inlineStr">
+        <is>
+          <t>Application viewed 6 days ago; recruiter active 1 day ago.</t>
+        </is>
+      </c>
+      <c r="O167" s="35" t="inlineStr">
+        <is>
+          <t>Active - Viewed</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="33.95" customHeight="1" s="20">
+      <c r="A168" s="35" t="inlineStr">
+        <is>
+          <t>Sep 01, 2026</t>
+        </is>
+      </c>
+      <c r="B168" s="36" t="inlineStr">
+        <is>
+          <t>Technology Cue</t>
+        </is>
+      </c>
+      <c r="C168" s="36" t="inlineStr">
+        <is>
+          <t>Senior Microsoft Fabric &amp; BI Solution Architect</t>
+        </is>
+      </c>
+      <c r="D168" s="36" t="inlineStr">
+        <is>
+          <t>Bangalore / Remote</t>
+        </is>
+      </c>
+      <c r="E168" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F168" s="35" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G168" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H168" s="35" t="inlineStr">
+        <is>
+          <t>Resume Viewed</t>
+        </is>
+      </c>
+      <c r="I168" s="36" t="inlineStr">
+        <is>
+          <t>Hiring Team</t>
+        </is>
+      </c>
+      <c r="J168" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K168" s="36" t="inlineStr">
+        <is>
+          <t>Resume Review</t>
+        </is>
+      </c>
+      <c r="L168" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M168" s="36" t="inlineStr">
+        <is>
+          <t>16-18 LPA</t>
+        </is>
+      </c>
+      <c r="N168" s="36" t="inlineStr">
+        <is>
+          <t>Resume viewed 6 days ago; recruiter active 3 days ago.</t>
+        </is>
+      </c>
+      <c r="O168" s="35" t="inlineStr">
+        <is>
+          <t>Active - Viewed</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="33.95" customHeight="1" s="20">
+      <c r="A169" s="35" t="inlineStr">
+        <is>
+          <t>Sep 01, 2026</t>
+        </is>
+      </c>
+      <c r="B169" s="36" t="inlineStr">
+        <is>
+          <t>Oaktree Capital Management</t>
+        </is>
+      </c>
+      <c r="C169" s="36" t="inlineStr">
+        <is>
+          <t>Risk, Reporting &amp; Analytics-Tech</t>
+        </is>
+      </c>
+      <c r="D169" s="36" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="E169" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F169" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G169" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H169" s="35" t="inlineStr">
+        <is>
+          <t>Application Sent</t>
+        </is>
+      </c>
+      <c r="I169" s="36" t="inlineStr">
+        <is>
+          <t>Recruiter Team</t>
+        </is>
+      </c>
+      <c r="J169" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K169" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L169" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M169" s="36" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N169" s="36" t="inlineStr">
+        <is>
+          <t>Application sent 5 days ago; recruiter active 4 days ago.</t>
+        </is>
+      </c>
+      <c r="O169" s="35" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="33.95" customHeight="1" s="20">
+      <c r="A170" s="35" t="inlineStr">
+        <is>
+          <t>Sep 02, 2026</t>
+        </is>
+      </c>
+      <c r="B170" s="36" t="inlineStr">
+        <is>
+          <t>Alike Thoughts</t>
+        </is>
+      </c>
+      <c r="C170" s="36" t="inlineStr">
+        <is>
+          <t>Data Architect / Lead</t>
+        </is>
+      </c>
+      <c r="D170" s="36" t="inlineStr">
+        <is>
+          <t>Pune / Remote</t>
+        </is>
+      </c>
+      <c r="E170" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F170" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G170" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H170" s="35" t="inlineStr">
+        <is>
+          <t>Application Sent</t>
+        </is>
+      </c>
+      <c r="I170" s="36" t="inlineStr">
+        <is>
+          <t>Sanika Sankpal</t>
+        </is>
+      </c>
+      <c r="J170" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K170" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L170" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M170" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N170" s="36" t="inlineStr">
+        <is>
+          <t>Application sent; contact unlocked on Naukri.</t>
+        </is>
+      </c>
+      <c r="O170" s="35" t="inlineStr">
+        <is>
+          <t>Active - In Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="33.95" customHeight="1" s="20">
+      <c r="A171" s="35" t="inlineStr">
+        <is>
+          <t>Sep 02, 2026</t>
+        </is>
+      </c>
+      <c r="B171" s="36" t="inlineStr">
+        <is>
+          <t>Saguna Consulting Services</t>
+        </is>
+      </c>
+      <c r="C171" s="36" t="inlineStr">
+        <is>
+          <t>Power BI Developer</t>
+        </is>
+      </c>
+      <c r="D171" s="36" t="inlineStr">
+        <is>
+          <t>Bangalore / Remote</t>
+        </is>
+      </c>
+      <c r="E171" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F171" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G171" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H171" s="35" t="inlineStr">
+        <is>
+          <t>Application Sent</t>
+        </is>
+      </c>
+      <c r="I171" s="36" t="inlineStr">
+        <is>
+          <t>HR Team</t>
+        </is>
+      </c>
+      <c r="J171" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K171" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L171" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M171" s="36" t="inlineStr">
+        <is>
+          <t>14-16 LPA</t>
+        </is>
+      </c>
+      <c r="N171" s="36" t="inlineStr">
+        <is>
+          <t>Application sent; Power BI and DAX reporting.</t>
+        </is>
+      </c>
+      <c r="O171" s="35" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="33.95" customHeight="1" s="20">
+      <c r="A172" s="35" t="inlineStr">
+        <is>
+          <t>Sep 02, 2026</t>
+        </is>
+      </c>
+      <c r="B172" s="36" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="C172" s="36" t="inlineStr">
+        <is>
+          <t>Data Modeller / Data Engineer</t>
+        </is>
+      </c>
+      <c r="D172" s="36" t="inlineStr">
+        <is>
+          <t>Pune / Bangalore</t>
+        </is>
+      </c>
+      <c r="E172" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F172" s="35" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G172" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H172" s="35" t="inlineStr">
+        <is>
+          <t>Application Sent</t>
+        </is>
+      </c>
+      <c r="I172" s="36" t="inlineStr">
+        <is>
+          <t>PO_1 (Sr HR)</t>
+        </is>
+      </c>
+      <c r="J172" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K172" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L172" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M172" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N172" s="36" t="inlineStr">
+        <is>
+          <t>Applied via NVite; recruiter active.</t>
+        </is>
+      </c>
+      <c r="O172" s="35" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="33.95" customHeight="1" s="20">
+      <c r="A173" s="35" t="inlineStr">
+        <is>
+          <t>Sep 02, 2026</t>
+        </is>
+      </c>
+      <c r="B173" s="36" t="inlineStr">
+        <is>
+          <t>Odiware Technologies</t>
+        </is>
+      </c>
+      <c r="C173" s="36" t="inlineStr">
+        <is>
+          <t>Snowflake Data Engineer (C2H)</t>
+        </is>
+      </c>
+      <c r="D173" s="36" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="E173" s="35" t="inlineStr">
+        <is>
+          <t>Naukri / Email</t>
+        </is>
+      </c>
+      <c r="F173" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G173" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Snowflake_Data_Engineer_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H173" s="35" t="inlineStr">
+        <is>
+          <t>Applied &amp; Resume Emailed</t>
+        </is>
+      </c>
+      <c r="I173" s="36" t="inlineStr">
+        <is>
+          <t>Usha Kiran P</t>
+        </is>
+      </c>
+      <c r="J173" s="36" t="inlineStr">
+        <is>
+          <t>Email / Naukri</t>
+        </is>
+      </c>
+      <c r="K173" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L173" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M173" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N173" s="36" t="inlineStr">
+        <is>
+          <t>Applied on Naukri and delivered tailored resume directly to recruiter.</t>
+        </is>
+      </c>
+      <c r="O173" s="35" t="inlineStr">
+        <is>
+          <t>Active - Resume Delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="33.95" customHeight="1" s="20">
+      <c r="A174" s="35" t="inlineStr">
+        <is>
+          <t>Sep 07, 2026</t>
+        </is>
+      </c>
+      <c r="B174" s="36" t="inlineStr">
+        <is>
+          <t>Cygnus Professionals</t>
+        </is>
+      </c>
+      <c r="C174" s="36" t="inlineStr">
+        <is>
+          <t>Data Modeler (Fabric Lakehouse)</t>
+        </is>
+      </c>
+      <c r="D174" s="36" t="inlineStr">
+        <is>
+          <t>Hyderabad / Remote</t>
+        </is>
+      </c>
+      <c r="E174" s="35" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="F174" s="35" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G174" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H174" s="35" t="inlineStr">
+        <is>
+          <t>Resume Viewed 1d Ago</t>
+        </is>
+      </c>
+      <c r="I174" s="36" t="inlineStr">
+        <is>
+          <t>Manasa Rapalli</t>
+        </is>
+      </c>
+      <c r="J174" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K174" s="36" t="inlineStr">
+        <is>
+          <t>Resume Review</t>
+        </is>
+      </c>
+      <c r="L174" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M174" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N174" s="36" t="inlineStr">
+        <is>
+          <t>Applied with honest screening (Schema Design: 10, Metadata: 8); resume viewed within 40 mins.</t>
+        </is>
+      </c>
+      <c r="O174" s="35" t="inlineStr">
+        <is>
+          <t>Active - Warm View</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="33.95" customHeight="1" s="20">
+      <c r="A175" s="35" t="inlineStr">
+        <is>
+          <t>Sep 07, 2026</t>
+        </is>
+      </c>
+      <c r="B175" s="36" t="inlineStr">
+        <is>
+          <t>EVERSANA</t>
+        </is>
+      </c>
+      <c r="C175" s="36" t="inlineStr">
+        <is>
+          <t>Power BI Developer (Fabric &amp; D365)</t>
+        </is>
+      </c>
+      <c r="D175" s="36" t="inlineStr">
+        <is>
+          <t>100% Remote India</t>
+        </is>
+      </c>
+      <c r="E175" s="35" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct</t>
+        </is>
+      </c>
+      <c r="F175" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G175" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H175" s="35" t="inlineStr">
+        <is>
+          <t>Resume Delivered to TA Lead</t>
+        </is>
+      </c>
+      <c r="I175" s="36" t="inlineStr">
+        <is>
+          <t>Mustafa Dhariwala</t>
+        </is>
+      </c>
+      <c r="J175" s="36" t="inlineStr">
+        <is>
+          <t>LinkedIn Chat</t>
+        </is>
+      </c>
+      <c r="K175" s="36" t="inlineStr">
+        <is>
+          <t>TA Review</t>
+        </is>
+      </c>
+      <c r="L175" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M175" s="36" t="inlineStr">
+        <is>
+          <t>15-18 LPA</t>
+        </is>
+      </c>
+      <c r="N175" s="36" t="inlineStr">
+        <is>
+          <t>1st-degree connection established; tailored resume and pitch delivered directly in chat.</t>
+        </is>
+      </c>
+      <c r="O175" s="35" t="inlineStr">
+        <is>
+          <t>Active - In Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="33.95" customHeight="1" s="20">
+      <c r="A176" s="35" t="inlineStr">
+        <is>
+          <t>Sep 07, 2026</t>
+        </is>
+      </c>
+      <c r="B176" s="36" t="inlineStr">
+        <is>
+          <t>KMK Consulting Inc. / Tredence</t>
+        </is>
+      </c>
+      <c r="C176" s="36" t="inlineStr">
+        <is>
+          <t>Manager Data Management</t>
+        </is>
+      </c>
+      <c r="D176" s="36" t="inlineStr">
+        <is>
+          <t>100% Remote India</t>
+        </is>
+      </c>
+      <c r="E176" s="35" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply</t>
+        </is>
+      </c>
+      <c r="F176" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G176" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H176" s="35" t="inlineStr">
+        <is>
+          <t>Applied - InMail Delivered</t>
+        </is>
+      </c>
+      <c r="I176" s="36" t="inlineStr">
+        <is>
+          <t>Pratik Salunke</t>
+        </is>
+      </c>
+      <c r="J176" s="36" t="inlineStr">
+        <is>
+          <t>LinkedIn InMail</t>
+        </is>
+      </c>
+      <c r="K176" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L176" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M176" s="36" t="inlineStr">
+        <is>
+          <t>18-22 LPA</t>
+        </is>
+      </c>
+      <c r="N176" s="36" t="inlineStr">
+        <is>
+          <t>Applied with 100% honest screening numbers (12y MDM, 7y ETL, 8y Team Lead); direct InMail sent to hiring lead.</t>
+        </is>
+      </c>
+      <c r="O176" s="35" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="33.95" customHeight="1" s="20">
+      <c r="A177" s="35" t="inlineStr">
+        <is>
+          <t>Sep 08, 2026</t>
+        </is>
+      </c>
+      <c r="B177" s="36" t="inlineStr">
+        <is>
+          <t>Vergil Remnant Consultant Services</t>
+        </is>
+      </c>
+      <c r="C177" s="36" t="inlineStr">
+        <is>
+          <t>Analytics Lead / BI Consultant</t>
+        </is>
+      </c>
+      <c r="D177" s="36" t="inlineStr">
+        <is>
+          <t>100% Remote India</t>
+        </is>
+      </c>
+      <c r="E177" s="35" t="inlineStr">
+        <is>
+          <t>Naukri NVite</t>
+        </is>
+      </c>
+      <c r="F177" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G177" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H177" s="35" t="inlineStr">
+        <is>
+          <t>Application Viewed Today</t>
+        </is>
+      </c>
+      <c r="I177" s="36" t="inlineStr">
+        <is>
+          <t>Prasad / Abhilash</t>
+        </is>
+      </c>
+      <c r="J177" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K177" s="36" t="inlineStr">
+        <is>
+          <t>Application Review</t>
+        </is>
+      </c>
+      <c r="L177" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M177" s="36" t="inlineStr">
+        <is>
+          <t>16-18 LPA</t>
+        </is>
+      </c>
+      <c r="N177" s="36" t="inlineStr">
+        <is>
+          <t>Applied via NVite; recruiter actively reviewed application today.</t>
+        </is>
+      </c>
+      <c r="O177" s="35" t="inlineStr">
+        <is>
+          <t>Active - Hot Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="33.95" customHeight="1" s="20">
+      <c r="A178" s="35" t="inlineStr">
+        <is>
+          <t>Sep 08, 2026</t>
+        </is>
+      </c>
+      <c r="B178" s="36" t="inlineStr">
+        <is>
+          <t>Vergil Remnant Consultant Services</t>
+        </is>
+      </c>
+      <c r="C178" s="36" t="inlineStr">
+        <is>
+          <t>Semantic Modelling Specialist</t>
+        </is>
+      </c>
+      <c r="D178" s="36" t="inlineStr">
+        <is>
+          <t>100% Remote India</t>
+        </is>
+      </c>
+      <c r="E178" s="35" t="inlineStr">
+        <is>
+          <t>Naukri NVite</t>
+        </is>
+      </c>
+      <c r="F178" s="35" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G178" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H178" s="35" t="inlineStr">
+        <is>
+          <t>Application Sent Today</t>
+        </is>
+      </c>
+      <c r="I178" s="36" t="inlineStr">
+        <is>
+          <t>Prasad</t>
+        </is>
+      </c>
+      <c r="J178" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K178" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L178" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M178" s="36" t="inlineStr">
+        <is>
+          <t>16-18 LPA</t>
+        </is>
+      </c>
+      <c r="N178" s="36" t="inlineStr">
+        <is>
+          <t>Applied via NVite; high match for dimensional Star Schema modeling.</t>
+        </is>
+      </c>
+      <c r="O178" s="35" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="33.95" customHeight="1" s="20">
+      <c r="A179" s="35" t="inlineStr">
+        <is>
+          <t>Sep 08, 2026</t>
+        </is>
+      </c>
+      <c r="B179" s="36" t="inlineStr">
+        <is>
+          <t>Quess Corp</t>
+        </is>
+      </c>
+      <c r="C179" s="36" t="inlineStr">
+        <is>
+          <t>Product Owner (Data Analytics &amp; ETL)</t>
+        </is>
+      </c>
+      <c r="D179" s="36" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad</t>
+        </is>
+      </c>
+      <c r="E179" s="35" t="inlineStr">
+        <is>
+          <t>Naukri NVite</t>
+        </is>
+      </c>
+      <c r="F179" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G179" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H179" s="35" t="inlineStr">
+        <is>
+          <t>Applied - NVite Linked</t>
+        </is>
+      </c>
+      <c r="I179" s="36" t="inlineStr">
+        <is>
+          <t>Sahithi M</t>
+        </is>
+      </c>
+      <c r="J179" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K179" s="36" t="inlineStr">
+        <is>
+          <t>Screening</t>
+        </is>
+      </c>
+      <c r="L179" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M179" s="36" t="inlineStr">
+        <is>
+          <t>16-20 LPA</t>
+        </is>
+      </c>
+      <c r="N179" s="36" t="inlineStr">
+        <is>
+          <t>CRITICAL CLAUSE: Requisition explicitly states Graduation Not Required! Status confirmed Applied.</t>
+        </is>
+      </c>
+      <c r="O179" s="35" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="33.95" customHeight="1" s="20">
+      <c r="A180" s="35" t="inlineStr">
+        <is>
+          <t>Sep 08, 2026</t>
+        </is>
+      </c>
+      <c r="B180" s="36" t="inlineStr">
+        <is>
+          <t>Datavail</t>
+        </is>
+      </c>
+      <c r="C180" s="36" t="inlineStr">
+        <is>
+          <t>Technical Specialist (Power BI &amp; Fabric)</t>
+        </is>
+      </c>
+      <c r="D180" s="36" t="inlineStr">
+        <is>
+          <t>Bengaluru / Mumbai / Hyderabad</t>
+        </is>
+      </c>
+      <c r="E180" s="35" t="inlineStr">
+        <is>
+          <t>Naukri NVite</t>
+        </is>
+      </c>
+      <c r="F180" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G180" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H180" s="35" t="inlineStr">
+        <is>
+          <t>Applied &amp; NVite Linked</t>
+        </is>
+      </c>
+      <c r="I180" s="36" t="inlineStr">
+        <is>
+          <t>Shirin Rafi</t>
+        </is>
+      </c>
+      <c r="J180" s="36" t="inlineStr">
+        <is>
+          <t>Naukri Portal</t>
+        </is>
+      </c>
+      <c r="K180" s="36" t="inlineStr">
+        <is>
+          <t>Candidate Folder</t>
+        </is>
+      </c>
+      <c r="L180" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M180" s="36" t="inlineStr">
+        <is>
+          <t>16-18 LPA</t>
+        </is>
+      </c>
+      <c r="N180" s="36" t="inlineStr">
+        <is>
+          <t>Direct NVite received from HR Manager Shirin Rafi; screening completed (10y Data Modeling, 8y Dashboards). Aligns with published book.</t>
+        </is>
+      </c>
+      <c r="O180" s="35" t="inlineStr">
+        <is>
+          <t>Active - High Priority Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="33.95" customHeight="1" s="20">
+      <c r="A181" s="35" t="inlineStr">
+        <is>
+          <t>Sep 08, 2026</t>
+        </is>
+      </c>
+      <c r="B181" s="36" t="inlineStr">
+        <is>
+          <t>Newbie Soft Solutions (TCS Deployment)</t>
+        </is>
+      </c>
+      <c r="C181" s="36" t="inlineStr">
+        <is>
+          <t>Snowflake Data Engineer</t>
+        </is>
+      </c>
+      <c r="D181" s="36" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad</t>
+        </is>
+      </c>
+      <c r="E181" s="35" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Direct</t>
+        </is>
+      </c>
+      <c r="F181" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G181" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Snowflake_Data_Engineer_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H181" s="35" t="inlineStr">
+        <is>
+          <t>Screened - Submitted to TCS</t>
+        </is>
+      </c>
+      <c r="I181" s="36" t="inlineStr">
+        <is>
+          <t>Faritha Banu M &amp; Juniad</t>
+        </is>
+      </c>
+      <c r="J181" s="36" t="inlineStr">
+        <is>
+          <t>Phone: +91 8428043416</t>
+        </is>
+      </c>
+      <c r="K181" s="36" t="inlineStr">
+        <is>
+          <t>TCS Panel Review</t>
+        </is>
+      </c>
+      <c r="L181" s="35" t="inlineStr">
+        <is>
+          <t>Awaiting Slots</t>
+        </is>
+      </c>
+      <c r="M181" s="36" t="inlineStr">
+        <is>
+          <t>10L Current / 16L Expected</t>
+        </is>
+      </c>
+      <c r="N181" s="36" t="inlineStr">
+        <is>
+          <t>Screened via live phone call at 1:00 PM; 3y Snowflake and 16L CTC confirmed; email acknowledgment and resume submitted; WhatsApp alert delivered.</t>
+        </is>
+      </c>
+      <c r="O181" s="35" t="inlineStr">
+        <is>
+          <t>Active - Interview Scheduled Stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="33.95" customHeight="1" s="20">
+      <c r="A182" s="35" t="inlineStr">
+        <is>
+          <t>Sep 08, 2026</t>
+        </is>
+      </c>
+      <c r="B182" s="36" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet</t>
+        </is>
+      </c>
+      <c r="C182" s="36" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer (Job # 11476)</t>
+        </is>
+      </c>
+      <c r="D182" s="36" t="inlineStr">
+        <is>
+          <t>Bengaluru (Hybrid - 3d in office)</t>
+        </is>
+      </c>
+      <c r="E182" s="35" t="inlineStr">
+        <is>
+          <t>Official Careers Portal</t>
+        </is>
+      </c>
+      <c r="F182" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G182" s="36" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Snowflake_Data_Engineer_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H182" s="35" t="inlineStr">
+        <is>
+          <t>Applied - Official Portal Submitted</t>
+        </is>
+      </c>
+      <c r="I182" s="36" t="inlineStr">
+        <is>
+          <t>Corporate Talent Team</t>
+        </is>
+      </c>
+      <c r="J182" s="36" t="inlineStr">
+        <is>
+          <t>careers.zimmerbiomet.com</t>
+        </is>
+      </c>
+      <c r="K182" s="36" t="inlineStr">
+        <is>
+          <t>Application Submitted</t>
+        </is>
+      </c>
+      <c r="L182" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M182" s="36" t="inlineStr">
+        <is>
+          <t>INR 16,00,000 Expected</t>
+        </is>
+      </c>
+      <c r="N182" s="36" t="inlineStr">
+        <is>
+          <t>Global med-tech leader; 11 AM - 8 PM shift; Snowflake, SQL pipelines, Medallion, CDC, data governance. Full honest disclosure (NIOS).</t>
+        </is>
+      </c>
+      <c r="O182" s="35" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
     <row r="183" ht="33.95" customHeight="1" s="20"/>
     <row r="184" ht="33.95" customHeight="1" s="20"/>
     <row r="185" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
docs: add Pillar 2 DAX VertiPaq Performance Optimization Interview Mastery guide and sync tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -769,7 +769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O182"/>
+  <dimension ref="A1:O185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -13501,9 +13501,237 @@
         </is>
       </c>
     </row>
-    <row r="183" ht="33.95" customHeight="1" s="20"/>
-    <row r="184" ht="33.95" customHeight="1" s="20"/>
-    <row r="185" ht="33.95" customHeight="1" s="20"/>
+    <row r="183" ht="33.95" customHeight="1" s="20">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>JOB-203</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Networth Corp</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>BI Specialist / Data Visualization Lead (IBCS)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>India (Remote)</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>18.0 - 25.0 LPA</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply (Job ID: 4467844884)</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Applied - Under Review</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Hiring Team (Networth Corp)</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Remote / LinkedIn Portal</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Submitted with published author credential ("The Comprehensive Power BI Handbook" on Amazon), DAX Studio / VertiPaq tuning, 15 days notice, 18 LPA expected.</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>18,00,000 LPA (Entered in Portal)</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>100% Remote. Boutique IBCS data visualization consulting. Fits Bloomberg-style visual restraint, DAX calculation groups, and financial reporting background.</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="33.95" customHeight="1" s="20">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>JOB-204</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Alkemiz Pty Ltd</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Fabric Data Lead (Lakehouse, DAX &amp; Governance)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Remote (India)</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>18.0 - 25.0 LPA</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply (Job ID: 4467855388)</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Applied - Under Review</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Garima Sharma (Lead Recruiter)</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>garima.sharma@alkemiz.com.au</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Urgent hiring! Confirmed immediate joining availability, 14.5 yrs experience, Medallion Lakehouse architecture, and Power BI Amazon published author.</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>18 LPA (Entered in Portal)</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>Australian retail IT services firm. 100% remote. Roles manages Fabric capacity, OneLake, Power BI semantic models, and DataOps. Direct recruiter email available.</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="33.95" customHeight="1" s="20">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>JOB-205</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Mphasis</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Business Analyst - Payment Domain (Data Reconciliation &amp; Analytics)</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>8.0 - 18.0 LPA</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Naukri (Job ID: 190926016406) + Direct Recruiter Email</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Applied - Direct Recruiter Contacted</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Reena Kumari (Mphasis Talent Acquisition)</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>reena.kumari@mphasis.com</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Applied on Naukri just after posting + sent personalized email with Form 16 verification, 3-tier financial reconciliation framework, and 15 days notice.</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>16.0 - 18.0 LPA Target</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>Payment Domain analytics. Matches 14.5 yrs data operations, financial reconciliation between upstream billing &amp; reporting marts, and live portfolio simulator.</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>Active - Under Review</t>
+        </is>
+      </c>
+    </row>
     <row r="186" ht="33.95" customHeight="1" s="20"/>
     <row r="187" ht="33.95" customHeight="1" s="20"/>
     <row r="188" ht="33.95" customHeight="1" s="20"/>

</xml_diff>